<commit_message>
update notebook with demo and add documentation
</commit_message>
<xml_diff>
--- a/exp_templates/Demo_Results_formulation_sheet.xlsx
+++ b/exp_templates/Demo_Results_formulation_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livejohnshopkins-my.sharepoint.com/personal/wtoh2_jh_edu/Documents/Research/falcon-lnp-optimization-LIVE/exp_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_89BDD6BA4E98484B49A7382031F91AA1ADA60D68" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="11_89BDD6BA4E98484B49173479A95E17F9ADA60CB5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB95C0CC-DC7D-47A3-B793-41D4AE91A1C8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2946,76 +2946,76 @@
       </c>
       <c r="B10" s="116"/>
       <c r="C10" s="101">
-        <v>14.173</v>
+        <v>4.8789999999999996</v>
       </c>
       <c r="D10" s="101">
-        <v>16.97</v>
+        <v>16.658999999999999</v>
       </c>
       <c r="E10" s="101">
-        <v>9.1289999999999996</v>
+        <v>14.336</v>
       </c>
       <c r="F10" s="101">
-        <v>18.728999999999999</v>
+        <v>8.7739999999999991</v>
       </c>
       <c r="G10" s="101">
-        <v>16.765999999999998</v>
+        <v>8.2240000000000002</v>
       </c>
       <c r="H10" s="101">
-        <v>16.387</v>
+        <v>18.542000000000002</v>
       </c>
       <c r="I10" s="101">
-        <v>9.8420000000000005</v>
+        <v>15.654</v>
       </c>
       <c r="J10" s="101">
-        <v>7.7</v>
+        <v>8.91</v>
       </c>
       <c r="K10" s="101">
-        <v>7.5759999999999996</v>
+        <v>17.192</v>
       </c>
       <c r="L10" s="101">
-        <v>20</v>
+        <v>13.672000000000001</v>
       </c>
       <c r="M10" s="101">
-        <v>15.856</v>
+        <v>12.47</v>
       </c>
       <c r="N10" s="101">
-        <v>7.2119999999999997</v>
+        <v>14.471</v>
       </c>
       <c r="O10" s="101">
-        <v>3.7570000000000001</v>
+        <v>2.673</v>
       </c>
       <c r="P10" s="101">
-        <v>2.621</v>
+        <v>4.4589999999999996</v>
       </c>
       <c r="Q10" s="101">
-        <v>4.4889999999999999</v>
+        <v>2.2290000000000001</v>
       </c>
       <c r="R10" s="101">
-        <v>2.0840000000000001</v>
+        <v>6.7089999999999996</v>
       </c>
       <c r="S10" s="101">
-        <v>5.8280000000000003</v>
+        <v>4.0289999999999999</v>
       </c>
       <c r="T10" s="101">
-        <v>6.7039999999999997</v>
+        <v>3.03</v>
       </c>
       <c r="U10" s="101">
-        <v>4.923</v>
+        <v>10.419</v>
       </c>
       <c r="V10" s="101">
-        <v>14.496</v>
+        <v>6.601</v>
       </c>
       <c r="W10" s="101">
-        <v>15.96</v>
+        <v>13.696</v>
       </c>
       <c r="X10" s="101">
-        <v>12.432</v>
+        <v>19.495999999999999</v>
       </c>
       <c r="Y10" s="101">
-        <v>15.292</v>
+        <v>8.1389999999999993</v>
       </c>
       <c r="Z10" s="101">
-        <v>17.524000000000001</v>
+        <v>11.755000000000001</v>
       </c>
       <c r="AA10" s="101"/>
       <c r="AB10" s="101"/>
@@ -3138,76 +3138,76 @@
       </c>
       <c r="B11" s="116"/>
       <c r="C11" s="101">
-        <v>51.338999999999999</v>
+        <v>51.87</v>
       </c>
       <c r="D11" s="101">
-        <v>54.545999999999999</v>
+        <v>52.994</v>
       </c>
       <c r="E11" s="101">
-        <v>53.886000000000003</v>
+        <v>53.683</v>
       </c>
       <c r="F11" s="101">
-        <v>55.689</v>
+        <v>56.988</v>
       </c>
       <c r="G11" s="101">
-        <v>52.594000000000001</v>
+        <v>54.170999999999999</v>
       </c>
       <c r="H11" s="101">
-        <v>55.378999999999998</v>
+        <v>53.991999999999997</v>
       </c>
       <c r="I11" s="101">
-        <v>53.680999999999997</v>
+        <v>43.472000000000001</v>
       </c>
       <c r="J11" s="101">
-        <v>53.551000000000002</v>
+        <v>52.279000000000003</v>
       </c>
       <c r="K11" s="101">
-        <v>58.573</v>
+        <v>52.143999999999998</v>
       </c>
       <c r="L11" s="101">
-        <v>54.731999999999999</v>
+        <v>53.994999999999997</v>
       </c>
       <c r="M11" s="101">
-        <v>54.51</v>
+        <v>58.500999999999998</v>
       </c>
       <c r="N11" s="101">
-        <v>53.14</v>
+        <v>53.850999999999999</v>
       </c>
       <c r="O11" s="101">
-        <v>83.292000000000002</v>
+        <v>78.072000000000003</v>
       </c>
       <c r="P11" s="101">
-        <v>65.168999999999997</v>
+        <v>51.838000000000001</v>
       </c>
       <c r="Q11" s="101">
-        <v>64.992999999999995</v>
+        <v>63.405000000000001</v>
       </c>
       <c r="R11" s="101">
-        <v>66.954999999999998</v>
+        <v>51.835999999999999</v>
       </c>
       <c r="S11" s="101">
-        <v>65.186000000000007</v>
+        <v>51.844999999999999</v>
       </c>
       <c r="T11" s="101">
-        <v>62.088999999999999</v>
+        <v>79.873999999999995</v>
       </c>
       <c r="U11" s="101">
-        <v>26.962</v>
+        <v>55.796999999999997</v>
       </c>
       <c r="V11" s="101">
-        <v>50.094000000000001</v>
+        <v>34.433999999999997</v>
       </c>
       <c r="W11" s="101">
-        <v>36.177</v>
+        <v>59.448</v>
       </c>
       <c r="X11" s="101">
-        <v>42.962000000000003</v>
+        <v>39.468000000000004</v>
       </c>
       <c r="Y11" s="101">
-        <v>87.757000000000005</v>
+        <v>77.421000000000006</v>
       </c>
       <c r="Z11" s="101">
-        <v>89.304000000000002</v>
+        <v>78.655000000000001</v>
       </c>
       <c r="AA11" s="101"/>
       <c r="AB11" s="101"/>
@@ -3330,76 +3330,76 @@
       </c>
       <c r="B12" s="116"/>
       <c r="C12" s="101">
-        <v>21.574999999999999</v>
+        <v>23.084</v>
       </c>
       <c r="D12" s="101">
-        <v>19.331</v>
+        <v>26.263999999999999</v>
       </c>
       <c r="E12" s="101">
-        <v>26.503</v>
+        <v>18.414999999999999</v>
       </c>
       <c r="F12" s="101">
-        <v>24.824999999999999</v>
+        <v>25.143999999999998</v>
       </c>
       <c r="G12" s="101">
-        <v>26.952000000000002</v>
+        <v>20.609000000000002</v>
       </c>
       <c r="H12" s="101">
-        <v>23.574000000000002</v>
+        <v>26.113</v>
       </c>
       <c r="I12" s="101">
-        <v>65.798000000000002</v>
+        <v>22.949000000000002</v>
       </c>
       <c r="J12" s="101">
-        <v>19.466999999999999</v>
+        <v>49.853999999999999</v>
       </c>
       <c r="K12" s="101">
-        <v>26.033999999999999</v>
+        <v>53.097999999999999</v>
       </c>
       <c r="L12" s="101">
-        <v>26.56</v>
+        <v>46.223999999999997</v>
       </c>
       <c r="M12" s="101">
-        <v>39.936999999999998</v>
+        <v>26.274000000000001</v>
       </c>
       <c r="N12" s="101">
-        <v>43.905999999999999</v>
+        <v>59.305</v>
       </c>
       <c r="O12" s="101">
-        <v>0.379</v>
+        <v>0.16900000000000001</v>
       </c>
       <c r="P12" s="101">
-        <v>1.0609999999999999</v>
+        <v>79.915999999999997</v>
       </c>
       <c r="Q12" s="101">
-        <v>60.362000000000002</v>
+        <v>5.3999999999999999E-2</v>
       </c>
       <c r="R12" s="101">
-        <v>0.108</v>
+        <v>79.69</v>
       </c>
       <c r="S12" s="101">
-        <v>79.393000000000001</v>
+        <v>59.058999999999997</v>
       </c>
       <c r="T12" s="101">
-        <v>75.772000000000006</v>
+        <v>0.58599999999999997</v>
       </c>
       <c r="U12" s="101">
-        <v>13.446999999999999</v>
+        <v>40.768999999999998</v>
       </c>
       <c r="V12" s="101">
-        <v>76.872</v>
+        <v>13.347</v>
       </c>
       <c r="W12" s="101">
-        <v>36.531999999999996</v>
+        <v>57.311999999999998</v>
       </c>
       <c r="X12" s="101">
-        <v>8.4339999999999993</v>
+        <v>7.3019999999999996</v>
       </c>
       <c r="Y12" s="101">
-        <v>22.654</v>
+        <v>21.097000000000001</v>
       </c>
       <c r="Z12" s="101">
-        <v>19.747</v>
+        <v>39.082000000000001</v>
       </c>
       <c r="AA12" s="101"/>
       <c r="AB12" s="101"/>
@@ -3522,76 +3522,76 @@
       </c>
       <c r="B13" s="117"/>
       <c r="C13" s="101">
-        <v>3.9860000000000002</v>
+        <v>0.877</v>
       </c>
       <c r="D13" s="101">
-        <v>0.89500000000000002</v>
+        <v>2.8050000000000002</v>
       </c>
       <c r="E13" s="101">
-        <v>0.93500000000000005</v>
+        <v>0.66200000000000003</v>
       </c>
       <c r="F13" s="101">
-        <v>0.79800000000000004</v>
+        <v>3.18</v>
       </c>
       <c r="G13" s="101">
-        <v>1.3420000000000001</v>
+        <v>1.121</v>
       </c>
       <c r="H13" s="101">
-        <v>4.0919999999999996</v>
+        <v>3.4660000000000002</v>
       </c>
       <c r="I13" s="101">
-        <v>3.992</v>
+        <v>0.58799999999999997</v>
       </c>
       <c r="J13" s="101">
-        <v>3.1030000000000002</v>
+        <v>3.944</v>
       </c>
       <c r="K13" s="101">
-        <v>3.504</v>
+        <v>2.1150000000000002</v>
       </c>
       <c r="L13" s="101">
-        <v>4.4039999999999999</v>
+        <v>3.6629999999999998</v>
       </c>
       <c r="M13" s="101">
-        <v>0.86399999999999999</v>
+        <v>3.5059999999999998</v>
       </c>
       <c r="N13" s="101">
-        <v>3.1890000000000001</v>
+        <v>3.4489999999999998</v>
       </c>
       <c r="O13" s="101">
-        <v>18.096</v>
+        <v>9.7080000000000002</v>
       </c>
       <c r="P13" s="101">
-        <v>10.529</v>
+        <v>10.382</v>
       </c>
       <c r="Q13" s="101">
-        <v>10.529</v>
+        <v>19.843</v>
       </c>
       <c r="R13" s="101">
-        <v>18.844000000000001</v>
+        <v>3.9049999999999998</v>
       </c>
       <c r="S13" s="101">
-        <v>8.0670000000000002</v>
+        <v>8.3339999999999996</v>
       </c>
       <c r="T13" s="101">
-        <v>3.3340000000000001</v>
+        <v>18.173999999999999</v>
       </c>
       <c r="U13" s="101">
-        <v>0.53400000000000003</v>
+        <v>13.778</v>
       </c>
       <c r="V13" s="101">
-        <v>17.128</v>
+        <v>9.1029999999999998</v>
       </c>
       <c r="W13" s="101">
-        <v>15.132</v>
+        <v>18.117000000000001</v>
       </c>
       <c r="X13" s="101">
-        <v>15.894</v>
+        <v>4.1559999999999997</v>
       </c>
       <c r="Y13" s="101">
-        <v>5.8460000000000001</v>
+        <v>7.36</v>
       </c>
       <c r="Z13" s="101">
-        <v>6.1219999999999999</v>
+        <v>12.489000000000001</v>
       </c>
       <c r="AA13" s="101"/>
       <c r="AB13" s="101"/>
@@ -4746,99 +4746,99 @@
       </c>
       <c r="C18" s="75">
         <f t="shared" ref="C18:AH18" si="0">(1-(C12/100))/(C12/100)</f>
-        <v>3.6349942062572422</v>
+        <v>3.3320048518454346</v>
       </c>
       <c r="D18" s="55">
         <f t="shared" si="0"/>
-        <v>4.1730381252909838</v>
+        <v>2.8074931465123365</v>
       </c>
       <c r="E18" s="13">
         <f t="shared" si="0"/>
-        <v>2.7731577557257672</v>
+        <v>4.4303556882975839</v>
       </c>
       <c r="F18" s="12">
         <f t="shared" si="0"/>
-        <v>3.0281973816717023</v>
+        <v>2.9770919503658924</v>
       </c>
       <c r="G18" s="55">
         <f t="shared" si="0"/>
-        <v>2.7102997922232115</v>
+        <v>3.8522490174195734</v>
       </c>
       <c r="H18" s="55">
         <f t="shared" si="0"/>
-        <v>3.2419614829897343</v>
+        <v>2.8295102056446986</v>
       </c>
       <c r="I18" s="12">
         <f t="shared" si="0"/>
-        <v>0.51980303352685486</v>
+        <v>3.3574883437186802</v>
       </c>
       <c r="J18" s="55">
         <f t="shared" si="0"/>
-        <v>4.136898340781836</v>
+        <v>1.005857102740001</v>
       </c>
       <c r="K18" s="55">
         <f t="shared" si="0"/>
-        <v>2.8411308289160329</v>
+        <v>0.88331010584202796</v>
       </c>
       <c r="L18" s="12">
         <f t="shared" si="0"/>
-        <v>2.7650602409638552</v>
+        <v>1.1633783316026307</v>
       </c>
       <c r="M18" s="55">
         <f t="shared" si="0"/>
-        <v>1.5039437113453689</v>
+        <v>2.8060439978686151</v>
       </c>
       <c r="N18" s="55">
         <f t="shared" si="0"/>
-        <v>1.2775930396756707</v>
+        <v>0.68619846555939645</v>
       </c>
       <c r="O18" s="12">
         <f t="shared" si="0"/>
-        <v>262.85224274406335</v>
+        <v>590.71597633136093</v>
       </c>
       <c r="P18" s="55">
         <f t="shared" si="0"/>
-        <v>93.250706880301607</v>
+        <v>0.25131387957355228</v>
       </c>
       <c r="Q18" s="55">
         <f t="shared" si="0"/>
-        <v>0.65667141579139177</v>
+        <v>1850.851851851852</v>
       </c>
       <c r="R18" s="12">
         <f t="shared" si="0"/>
-        <v>924.92592592592598</v>
+        <v>0.25486259254611632</v>
       </c>
       <c r="S18" s="55">
         <f t="shared" si="0"/>
-        <v>0.25955688788684139</v>
+        <v>0.69322203220508316</v>
       </c>
       <c r="T18" s="55">
         <f t="shared" si="0"/>
-        <v>0.31974871984374165</v>
+        <v>169.64846416382252</v>
       </c>
       <c r="U18" s="12">
         <f t="shared" si="0"/>
-        <v>6.4366029597679795</v>
+        <v>1.4528440727022984</v>
       </c>
       <c r="V18" s="55">
         <f t="shared" si="0"/>
-        <v>0.30086377354563437</v>
+        <v>6.4923203716190905</v>
       </c>
       <c r="W18" s="55">
         <f t="shared" si="0"/>
-        <v>1.7373261797875836</v>
+        <v>0.74483528754885553</v>
       </c>
       <c r="X18" s="12">
         <f t="shared" si="0"/>
-        <v>10.856770215793219</v>
+        <v>12.694878115584771</v>
       </c>
       <c r="Y18" s="55">
         <f t="shared" si="0"/>
-        <v>3.4142314822989319</v>
+        <v>3.7400104280229414</v>
       </c>
       <c r="Z18" s="55">
         <f t="shared" si="0"/>
-        <v>4.064060363599534</v>
+        <v>1.5587226856353309</v>
       </c>
       <c r="AA18" s="55" t="e">
         <f t="shared" si="0"/>
@@ -5303,99 +5303,99 @@
       </c>
       <c r="C19" s="75">
         <f t="shared" ref="C19:AH19" si="5">(1-(C13/100))/(C13/100)</f>
-        <v>24.087807325639741</v>
+        <v>113.02508551881415</v>
       </c>
       <c r="D19" s="55">
         <f t="shared" si="5"/>
-        <v>110.73184357541899</v>
+        <v>34.650623885918002</v>
       </c>
       <c r="E19" s="13">
         <f t="shared" si="5"/>
-        <v>105.95187165775401</v>
+        <v>150.05740181268882</v>
       </c>
       <c r="F19" s="12">
         <f t="shared" si="5"/>
-        <v>124.31328320802004</v>
+        <v>30.446540880503143</v>
       </c>
       <c r="G19" s="55">
         <f t="shared" si="5"/>
-        <v>73.515648286140078</v>
+        <v>88.206066012488847</v>
       </c>
       <c r="H19" s="55">
         <f t="shared" si="5"/>
-        <v>23.437927663734119</v>
+        <v>27.851702250432773</v>
       </c>
       <c r="I19" s="12">
         <f t="shared" si="5"/>
-        <v>24.050100200400806</v>
+        <v>169.06802721088437</v>
       </c>
       <c r="J19" s="55">
         <f t="shared" si="5"/>
-        <v>31.226877215597806</v>
+        <v>24.35496957403651</v>
       </c>
       <c r="K19" s="55">
         <f t="shared" si="5"/>
-        <v>27.538812785388128</v>
+        <v>46.281323877068552</v>
       </c>
       <c r="L19" s="12">
         <f t="shared" si="5"/>
-        <v>21.706630336058133</v>
+        <v>26.300027300027306</v>
       </c>
       <c r="M19" s="55">
         <f t="shared" si="5"/>
-        <v>114.74074074074075</v>
+        <v>27.522532800912721</v>
       </c>
       <c r="N19" s="55">
         <f t="shared" si="5"/>
-        <v>30.357792411414234</v>
+        <v>27.993911278631487</v>
       </c>
       <c r="O19" s="12">
         <f t="shared" si="5"/>
-        <v>4.5260831122900083</v>
+        <v>9.3007828594973212</v>
       </c>
       <c r="P19" s="55">
         <f t="shared" si="5"/>
-        <v>8.4975781175800176</v>
+        <v>8.6320554806395684</v>
       </c>
       <c r="Q19" s="55">
         <f t="shared" si="5"/>
-        <v>8.4975781175800176</v>
+        <v>4.0395605503200125</v>
       </c>
       <c r="R19" s="12">
         <f t="shared" si="5"/>
-        <v>4.3067289322861377</v>
+        <v>24.608194622279129</v>
       </c>
       <c r="S19" s="55">
         <f t="shared" si="5"/>
-        <v>11.396181975951405</v>
+        <v>10.999040076793857</v>
       </c>
       <c r="T19" s="55">
         <f t="shared" si="5"/>
-        <v>28.994001199760046</v>
+        <v>4.5023660173874767</v>
       </c>
       <c r="U19" s="12">
         <f t="shared" si="5"/>
-        <v>186.26591760299624</v>
+        <v>6.257947452460443</v>
       </c>
       <c r="V19" s="55">
         <f t="shared" si="5"/>
-        <v>4.838393274170949</v>
+        <v>9.9853894320553671</v>
       </c>
       <c r="W19" s="55">
         <f t="shared" si="5"/>
-        <v>5.608511763150938</v>
+        <v>4.5196776508251917</v>
       </c>
       <c r="X19" s="12">
         <f t="shared" si="5"/>
-        <v>5.2916823958726562</v>
+        <v>23.061597690086622</v>
       </c>
       <c r="Y19" s="55">
         <f t="shared" si="5"/>
-        <v>16.105713308244955</v>
+        <v>12.586956521739131</v>
       </c>
       <c r="Z19" s="55">
         <f t="shared" si="5"/>
-        <v>15.33453119895459</v>
+        <v>7.0070462006565783</v>
       </c>
       <c r="AA19" s="55" t="e">
         <f t="shared" si="5"/>
@@ -10168,91 +10168,91 @@
       </c>
       <c r="C31" s="75">
         <f t="shared" ref="C31:AH31" si="10">C55/C23*1000</f>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="D31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="E31" s="13">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="F31" s="12">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="G31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="H31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="I31" s="12">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="J31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="K31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="L31" s="12">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="M31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="N31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="O31" s="12">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1.2655904928842176E-2</v>
       </c>
       <c r="P31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="Q31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1.2655904928842176E-2</v>
       </c>
       <c r="R31" s="12">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="S31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="T31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>0.12655904928842177</v>
       </c>
       <c r="U31" s="12">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="V31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="W31" s="55">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="X31" s="12">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>6.3279524644210872</v>
       </c>
       <c r="Y31" s="55">
         <f t="shared" si="10"/>
@@ -10728,91 +10728,91 @@
       </c>
       <c r="C32" s="78">
         <f t="shared" ref="C32:AH32" si="15">C54/C22*1000</f>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="D32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="E32" s="1">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="F32" s="15">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="G32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="H32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="I32" s="15">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="J32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="K32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="L32" s="15">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="M32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="N32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="O32" s="15">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="P32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>7.7870703483935264</v>
       </c>
       <c r="Q32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="R32" s="15">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>7.7870703483935264</v>
       </c>
       <c r="S32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="T32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="U32" s="15">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="V32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="W32" s="58">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="X32" s="15">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>23.361211045180582</v>
       </c>
       <c r="Y32" s="58">
         <f t="shared" si="15"/>
@@ -11288,91 +11288,91 @@
       </c>
       <c r="C33" s="78">
         <f t="shared" ref="C33:AH33" si="20">C56/C24*1000</f>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="D33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="E33" s="1">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="F33" s="15">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="G33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="H33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="I33" s="15">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="J33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="K33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="L33" s="15">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="M33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="N33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="O33" s="15">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>2.5862916198978931</v>
       </c>
       <c r="P33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="Q33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>2.5862916198978931</v>
       </c>
       <c r="R33" s="15">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="S33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="T33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>2.5862916198978931</v>
       </c>
       <c r="U33" s="15">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="V33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="W33" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>12.931458099489467</v>
       </c>
       <c r="X33" s="15">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>38.794374298468398</v>
       </c>
       <c r="Y33" s="58">
         <f t="shared" si="20"/>
@@ -11848,91 +11848,91 @@
       </c>
       <c r="C34" s="78">
         <f t="shared" ref="C34:AH34" si="25">C57/C25*1000</f>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E34" s="1">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="F34" s="15">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="H34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I34" s="15">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="J34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="K34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L34" s="15">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="M34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="N34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O34" s="15">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="P34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="Q34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R34" s="15">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="S34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="T34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="U34" s="15">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W34" s="58">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X34" s="15">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y34" s="58">
         <f t="shared" si="25"/>
@@ -12550,99 +12550,99 @@
       </c>
       <c r="C36" s="75">
         <f t="shared" ref="C36:AH36" si="30">C37*C26*C10*100/(C27*C41+C28*C44)</f>
-        <v>414.10039151522238</v>
+        <v>141.09311740890689</v>
       </c>
       <c r="D36" s="55">
         <f t="shared" si="30"/>
-        <v>466.67033329666702</v>
+        <v>471.53451334113294</v>
       </c>
       <c r="E36" s="13">
         <f t="shared" si="30"/>
-        <v>254.11980848457853</v>
+        <v>400.57373842743516</v>
       </c>
       <c r="F36" s="12">
         <f t="shared" si="30"/>
-        <v>504.47126003339986</v>
+        <v>230.9433564961044</v>
       </c>
       <c r="G36" s="55">
         <f t="shared" si="30"/>
-        <v>478.17241510438447</v>
+        <v>227.72332059589081</v>
       </c>
       <c r="H36" s="55">
         <f t="shared" si="30"/>
-        <v>443.85958576355659</v>
+        <v>515.13187138835383</v>
       </c>
       <c r="I36" s="12">
         <f t="shared" si="30"/>
-        <v>275.01350570965519</v>
+        <v>540.14078027235917</v>
       </c>
       <c r="J36" s="55">
         <f t="shared" si="30"/>
-        <v>215.68224683012454</v>
+        <v>255.64758315958608</v>
       </c>
       <c r="K36" s="55">
         <f t="shared" si="30"/>
-        <v>194.0143069332286</v>
+        <v>494.5535440319116</v>
       </c>
       <c r="L36" s="12">
         <f t="shared" si="30"/>
-        <v>548.12541109405834</v>
+        <v>379.81294564311509</v>
       </c>
       <c r="M36" s="55">
         <f t="shared" si="30"/>
-        <v>436.32361034672539</v>
+        <v>319.73812413463014</v>
       </c>
       <c r="N36" s="55">
         <f t="shared" si="30"/>
-        <v>203.57546104629282</v>
+        <v>403.08443668641252</v>
       </c>
       <c r="O36" s="12">
         <f t="shared" si="30"/>
-        <v>67.6595591413341</v>
+        <v>51.356440209037807</v>
       </c>
       <c r="P36" s="55">
         <f t="shared" si="30"/>
-        <v>60.327763200294633</v>
+        <v>129.02696863304911</v>
       </c>
       <c r="Q36" s="55">
         <f t="shared" si="30"/>
-        <v>103.60346498853723</v>
+        <v>52.732434350603263</v>
       </c>
       <c r="R36" s="12">
         <f t="shared" si="30"/>
-        <v>46.688074079605705</v>
+        <v>194.14113743344393</v>
       </c>
       <c r="S36" s="55">
         <f t="shared" si="30"/>
-        <v>134.10855091584079</v>
+        <v>116.56861799594947</v>
       </c>
       <c r="T36" s="55">
         <f t="shared" si="30"/>
-        <v>161.96105590362222</v>
+        <v>56.902120840323512</v>
       </c>
       <c r="U36" s="12">
         <f t="shared" si="30"/>
-        <v>273.88546843705956</v>
+        <v>280.09570407011125</v>
       </c>
       <c r="V36" s="55">
         <f t="shared" si="30"/>
-        <v>434.06395975565931</v>
+        <v>287.55009583551146</v>
       </c>
       <c r="W36" s="55">
         <f t="shared" si="30"/>
-        <v>661.74641346711996</v>
+        <v>345.57932983447716</v>
       </c>
       <c r="X36" s="12">
         <f t="shared" si="30"/>
-        <v>434.05800474838225</v>
+        <v>740.95469747643654</v>
       </c>
       <c r="Y36" s="55">
         <f t="shared" si="30"/>
-        <v>261.38085850701373</v>
+        <v>157.6897740923005</v>
       </c>
       <c r="Z36" s="55">
         <f t="shared" si="30"/>
-        <v>294.34291857027682</v>
+        <v>224.17519547390503</v>
       </c>
       <c r="AA36" s="55" t="e">
         <f t="shared" si="30"/>
@@ -14931,99 +14931,99 @@
       </c>
       <c r="C41" s="75">
         <f t="shared" ref="C41:AH41" si="50">C11*C18/(C18+1)</f>
-        <v>40.26261075</v>
+        <v>39.896329199999997</v>
       </c>
       <c r="D41" s="55">
         <f t="shared" si="50"/>
-        <v>44.001712740000002</v>
+        <v>39.075655840000003</v>
       </c>
       <c r="E41" s="13">
         <f t="shared" si="50"/>
-        <v>39.60459342</v>
+        <v>43.797275549999995</v>
       </c>
       <c r="F41" s="12">
         <f t="shared" si="50"/>
-        <v>41.864205749999996</v>
+        <v>42.658937279999996</v>
       </c>
       <c r="G41" s="55">
         <f t="shared" si="50"/>
-        <v>38.41886512</v>
+        <v>43.006898609999993</v>
       </c>
       <c r="H41" s="55">
         <f t="shared" si="50"/>
-        <v>42.323954539999995</v>
+        <v>39.89306904</v>
       </c>
       <c r="I41" s="12">
         <f t="shared" si="50"/>
-        <v>18.35997562</v>
+        <v>33.495610720000002</v>
       </c>
       <c r="J41" s="55">
         <f t="shared" si="50"/>
-        <v>43.12622683</v>
+        <v>26.215827340000001</v>
       </c>
       <c r="K41" s="55">
         <f t="shared" si="50"/>
-        <v>43.324105180000004</v>
+        <v>24.456578880000002</v>
       </c>
       <c r="L41" s="12">
         <f t="shared" si="50"/>
-        <v>40.195180799999996</v>
+        <v>29.036351200000002</v>
       </c>
       <c r="M41" s="55">
         <f t="shared" si="50"/>
-        <v>32.740341299999997</v>
+        <v>43.130447260000004</v>
       </c>
       <c r="N41" s="55">
         <f t="shared" si="50"/>
-        <v>29.808351600000002</v>
+        <v>21.914664450000004</v>
       </c>
       <c r="O41" s="12">
         <f t="shared" si="50"/>
-        <v>82.976323320000006</v>
+        <v>77.940058320000006</v>
       </c>
       <c r="P41" s="55">
         <f t="shared" si="50"/>
-        <v>64.47755690999999</v>
+        <v>10.411143920000002</v>
       </c>
       <c r="Q41" s="55">
         <f t="shared" si="50"/>
-        <v>25.761925339999994</v>
+        <v>63.370761299999998</v>
       </c>
       <c r="R41" s="12">
         <f t="shared" si="50"/>
-        <v>66.882688599999994</v>
+        <v>10.527891600000004</v>
       </c>
       <c r="S41" s="55">
         <f t="shared" si="50"/>
-        <v>13.432879020000003</v>
+        <v>21.225861450000004</v>
       </c>
       <c r="T41" s="55">
         <f t="shared" si="50"/>
-        <v>15.042922919999995</v>
+        <v>79.405938359999993</v>
       </c>
       <c r="U41" s="12">
         <f t="shared" si="50"/>
-        <v>23.336419859999999</v>
+        <v>33.049121070000005</v>
       </c>
       <c r="V41" s="55">
         <f t="shared" si="50"/>
-        <v>11.585740320000003</v>
+        <v>29.838094019999996</v>
       </c>
       <c r="W41" s="55">
         <f t="shared" si="50"/>
-        <v>22.960818360000001</v>
+        <v>25.377162240000004</v>
       </c>
       <c r="X41" s="12">
         <f t="shared" si="50"/>
-        <v>39.338584920000002</v>
+        <v>36.586046640000006</v>
       </c>
       <c r="Y41" s="55">
         <f t="shared" si="50"/>
-        <v>67.876529219999995</v>
+        <v>61.087491630000009</v>
       </c>
       <c r="Z41" s="55">
         <f t="shared" si="50"/>
-        <v>71.669139119999997</v>
+        <v>47.915052899999999</v>
       </c>
       <c r="AA41" s="55" t="e">
         <f t="shared" si="50"/>
@@ -15491,99 +15491,99 @@
       </c>
       <c r="C42" s="75">
         <f t="shared" ref="C42:AH42" si="55">C36*C41/100</f>
-        <v>166.72762875000001</v>
+        <v>56.290974599999998</v>
       </c>
       <c r="D42" s="55">
         <f t="shared" si="55"/>
-        <v>205.3429395</v>
+        <v>184.25520360000002</v>
       </c>
       <c r="E42" s="13">
         <f t="shared" si="55"/>
-        <v>100.64311694999998</v>
+        <v>175.44038399999997</v>
       </c>
       <c r="F42" s="12">
         <f t="shared" si="55"/>
-        <v>211.19288625000002</v>
+        <v>98.51798159999997</v>
       </c>
       <c r="G42" s="55">
         <f t="shared" si="55"/>
-        <v>183.70841519999999</v>
+        <v>97.936737600000001</v>
       </c>
       <c r="H42" s="55">
         <f t="shared" si="55"/>
-        <v>187.85892929999997</v>
+        <v>205.5019131</v>
       </c>
       <c r="I42" s="12">
         <f t="shared" si="55"/>
-        <v>50.492412599999994</v>
+        <v>180.92345310000002</v>
       </c>
       <c r="J42" s="55">
         <f t="shared" si="55"/>
-        <v>93.015614999999997</v>
+        <v>67.020129000000011</v>
       </c>
       <c r="K42" s="55">
         <f t="shared" si="55"/>
-        <v>84.054962400000008</v>
+        <v>120.9508776</v>
       </c>
       <c r="L42" s="12">
         <f t="shared" si="55"/>
-        <v>220.32</v>
+        <v>110.2838208</v>
       </c>
       <c r="M42" s="55">
         <f t="shared" si="55"/>
-        <v>142.85383920000001</v>
+        <v>137.904483</v>
       </c>
       <c r="N42" s="55">
         <f t="shared" si="55"/>
-        <v>60.682489200000006</v>
+        <v>88.334601750000019</v>
       </c>
       <c r="O42" s="12">
         <f t="shared" si="55"/>
-        <v>56.14141455</v>
+        <v>40.027239449999996</v>
       </c>
       <c r="P42" s="55">
         <f t="shared" si="55"/>
-        <v>38.897867850000004</v>
+        <v>13.433183400000003</v>
       </c>
       <c r="Q42" s="55">
         <f t="shared" si="55"/>
-        <v>26.690247299999992</v>
+        <v>33.4169451</v>
       </c>
       <c r="R42" s="12">
         <f t="shared" si="55"/>
-        <v>31.226239199999995</v>
+        <v>20.438968500000005</v>
       </c>
       <c r="S42" s="55">
         <f t="shared" si="55"/>
-        <v>18.0146394</v>
+        <v>24.742693350000003</v>
       </c>
       <c r="T42" s="55">
         <f t="shared" si="55"/>
-        <v>24.363676799999993</v>
+        <v>45.183662999999996</v>
       </c>
       <c r="U42" s="12">
         <f t="shared" si="55"/>
-        <v>63.915062849999998</v>
+        <v>92.569168349999998</v>
       </c>
       <c r="V42" s="55">
         <f t="shared" si="55"/>
-        <v>50.289523200000005</v>
+        <v>85.799467949999993</v>
       </c>
       <c r="W42" s="55">
         <f t="shared" si="55"/>
-        <v>151.94239200000001</v>
+        <v>87.698227200000005</v>
       </c>
       <c r="X42" s="12">
         <f t="shared" si="55"/>
-        <v>170.7522768</v>
+        <v>271.08603120000004</v>
       </c>
       <c r="Y42" s="55">
         <f t="shared" si="55"/>
-        <v>177.41625480000002</v>
+        <v>96.328727549999982</v>
       </c>
       <c r="Z42" s="55">
         <f t="shared" si="55"/>
-        <v>210.95303580000001</v>
+        <v>107.4136635</v>
       </c>
       <c r="AA42" s="55" t="e">
         <f t="shared" si="55"/>
@@ -16145,99 +16145,99 @@
       </c>
       <c r="C44" s="75">
         <f t="shared" ref="C44:AH44" si="60">C11/(1+C18)</f>
-        <v>11.07638925</v>
+        <v>11.973670799999997</v>
       </c>
       <c r="D44" s="55">
         <f t="shared" si="60"/>
-        <v>10.544287259999999</v>
+        <v>13.918344159999998</v>
       </c>
       <c r="E44" s="13">
         <f t="shared" si="60"/>
-        <v>14.281406580000001</v>
+        <v>9.8857244499999997</v>
       </c>
       <c r="F44" s="12">
         <f t="shared" si="60"/>
-        <v>13.824794249999997</v>
+        <v>14.32906272</v>
       </c>
       <c r="G44" s="55">
         <f t="shared" si="60"/>
-        <v>14.175134880000002</v>
+        <v>11.164101390000001</v>
       </c>
       <c r="H44" s="55">
         <f t="shared" si="60"/>
-        <v>13.055045460000001</v>
+        <v>14.098930959999997</v>
       </c>
       <c r="I44" s="12">
         <f t="shared" si="60"/>
-        <v>35.321024379999997</v>
+        <v>9.9763892800000011</v>
       </c>
       <c r="J44" s="55">
         <f t="shared" si="60"/>
-        <v>10.42477317</v>
+        <v>26.063172659999996</v>
       </c>
       <c r="K44" s="55">
         <f t="shared" si="60"/>
-        <v>15.24889482</v>
+        <v>27.68742112</v>
       </c>
       <c r="L44" s="12">
         <f t="shared" si="60"/>
-        <v>14.5368192</v>
+        <v>24.958648800000002</v>
       </c>
       <c r="M44" s="55">
         <f t="shared" si="60"/>
-        <v>21.769658700000001</v>
+        <v>15.370552740000001</v>
       </c>
       <c r="N44" s="55">
         <f t="shared" si="60"/>
-        <v>23.331648399999999</v>
+        <v>31.936335549999999</v>
       </c>
       <c r="O44" s="12">
         <f t="shared" si="60"/>
-        <v>0.31567667999999999</v>
+        <v>0.13194168000000001</v>
       </c>
       <c r="P44" s="55">
         <f t="shared" si="60"/>
-        <v>0.69144308999999993</v>
+        <v>41.42685608</v>
       </c>
       <c r="Q44" s="55">
         <f t="shared" si="60"/>
-        <v>39.231074660000004</v>
+        <v>3.4238699999999997E-2</v>
       </c>
       <c r="R44" s="12">
         <f t="shared" si="60"/>
-        <v>7.2311399999999998E-2</v>
+        <v>41.308108399999995</v>
       </c>
       <c r="S44" s="55">
         <f t="shared" si="60"/>
-        <v>51.753120980000013</v>
+        <v>30.619138549999999</v>
       </c>
       <c r="T44" s="55">
         <f t="shared" si="60"/>
-        <v>47.046077080000003</v>
+        <v>0.46806164</v>
       </c>
       <c r="U44" s="12">
         <f t="shared" si="60"/>
-        <v>3.6255801399999994</v>
+        <v>22.747878929999999</v>
       </c>
       <c r="V44" s="55">
         <f t="shared" si="60"/>
-        <v>38.508259680000002</v>
+        <v>4.5959059799999995</v>
       </c>
       <c r="W44" s="55">
         <f t="shared" si="60"/>
-        <v>13.21618164</v>
+        <v>34.070837759999996</v>
       </c>
       <c r="X44" s="12">
         <f t="shared" si="60"/>
-        <v>3.62341508</v>
+        <v>2.8819533600000002</v>
       </c>
       <c r="Y44" s="55">
         <f t="shared" si="60"/>
-        <v>19.88047078</v>
+        <v>16.333508370000004</v>
       </c>
       <c r="Z44" s="55">
         <f t="shared" si="60"/>
-        <v>17.634860880000002</v>
+        <v>30.739947099999998</v>
       </c>
       <c r="AA44" s="55" t="e">
         <f t="shared" si="60"/>
@@ -16705,99 +16705,99 @@
       </c>
       <c r="C45" s="75">
         <f t="shared" ref="C45:AH45" si="65">C36*C44/100</f>
-        <v>45.867371250000005</v>
+        <v>16.894025399999997</v>
       </c>
       <c r="D45" s="55">
         <f t="shared" si="65"/>
-        <v>49.207060499999997</v>
+        <v>65.629796399999989</v>
       </c>
       <c r="E45" s="13">
         <f t="shared" si="65"/>
-        <v>36.291883049999996</v>
+        <v>39.599615999999997</v>
       </c>
       <c r="F45" s="12">
         <f t="shared" si="65"/>
-        <v>69.742113749999987</v>
+        <v>33.092018399999994</v>
       </c>
       <c r="G45" s="55">
         <f t="shared" si="65"/>
-        <v>67.781584800000005</v>
+        <v>25.423262400000002</v>
       </c>
       <c r="H45" s="55">
         <f t="shared" si="65"/>
-        <v>57.9460707</v>
+        <v>72.628086899999985</v>
       </c>
       <c r="I45" s="12">
         <f t="shared" si="65"/>
-        <v>97.137587399999987</v>
+        <v>53.886546900000006</v>
       </c>
       <c r="J45" s="55">
         <f t="shared" si="65"/>
-        <v>22.484384999999996</v>
+        <v>66.629870999999994</v>
       </c>
       <c r="K45" s="55">
         <f t="shared" si="65"/>
-        <v>29.585037599999996</v>
+        <v>136.92912239999998</v>
       </c>
       <c r="L45" s="12">
         <f t="shared" si="65"/>
-        <v>79.680000000000007</v>
+        <v>94.796179200000012</v>
       </c>
       <c r="M45" s="55">
         <f t="shared" si="65"/>
-        <v>94.986160800000022</v>
+        <v>49.145516999999998</v>
       </c>
       <c r="N45" s="55">
         <f t="shared" si="65"/>
-        <v>47.497510800000001</v>
+        <v>128.73039825000001</v>
       </c>
       <c r="O45" s="12">
         <f t="shared" si="65"/>
-        <v>0.21358544999999998</v>
+        <v>6.7760549999999989E-2</v>
       </c>
       <c r="P45" s="55">
         <f t="shared" si="65"/>
-        <v>0.41713215000000003</v>
+        <v>53.451816600000001</v>
       </c>
       <c r="Q45" s="55">
         <f t="shared" si="65"/>
-        <v>40.644752700000005</v>
+        <v>1.8054899999999999E-2</v>
       </c>
       <c r="R45" s="12">
         <f t="shared" si="65"/>
-        <v>3.3760800000000001E-2</v>
+        <v>80.196031499999989</v>
       </c>
       <c r="S45" s="55">
         <f t="shared" si="65"/>
-        <v>69.405360600000009</v>
+        <v>35.692306649999999</v>
       </c>
       <c r="T45" s="55">
         <f t="shared" si="65"/>
-        <v>76.196323200000009</v>
+        <v>0.26633699999999999</v>
       </c>
       <c r="U45" s="12">
         <f t="shared" si="65"/>
-        <v>9.9299371499999989</v>
+        <v>63.715831649999991</v>
       </c>
       <c r="V45" s="55">
         <f t="shared" si="65"/>
-        <v>167.15047680000001</v>
+        <v>13.215532050000002</v>
       </c>
       <c r="W45" s="55">
         <f t="shared" si="65"/>
-        <v>87.457607999999993</v>
+        <v>117.74177279999998</v>
       </c>
       <c r="X45" s="12">
         <f t="shared" si="65"/>
-        <v>15.727723199999998</v>
+        <v>21.353968799999997</v>
       </c>
       <c r="Y45" s="55">
         <f t="shared" si="65"/>
-        <v>51.963745200000005</v>
+        <v>25.756272450000001</v>
       </c>
       <c r="Z45" s="55">
         <f t="shared" si="65"/>
-        <v>51.906964200000012</v>
+        <v>68.911336500000004</v>
       </c>
       <c r="AA45" s="55" t="e">
         <f t="shared" si="65"/>
@@ -17359,99 +17359,99 @@
       </c>
       <c r="C47" s="75">
         <f t="shared" ref="C47:AH47" si="70">(100-C11)*C19/(C19+1)</f>
-        <v>46.721372540000004</v>
+        <v>47.707899900000001</v>
       </c>
       <c r="D47" s="55">
         <f t="shared" si="70"/>
-        <v>45.047186699999997</v>
+        <v>45.687481699999999</v>
       </c>
       <c r="E47" s="13">
         <f t="shared" si="70"/>
-        <v>45.682834099999994</v>
+        <v>46.010381459999998</v>
       </c>
       <c r="F47" s="12">
         <f t="shared" si="70"/>
-        <v>43.957398220000002</v>
+        <v>41.6442184</v>
       </c>
       <c r="G47" s="55">
         <f t="shared" si="70"/>
-        <v>46.769811480000001</v>
+        <v>45.315256910000002</v>
       </c>
       <c r="H47" s="55">
         <f t="shared" si="70"/>
-        <v>42.795108679999998</v>
+        <v>44.413362720000002</v>
       </c>
       <c r="I47" s="12">
         <f t="shared" si="70"/>
-        <v>44.469945520000003</v>
+        <v>56.195615359999998</v>
       </c>
       <c r="J47" s="55">
         <f t="shared" si="70"/>
-        <v>45.007687529999991</v>
+        <v>45.838883759999995</v>
       </c>
       <c r="K47" s="55">
         <f t="shared" si="70"/>
-        <v>39.975397919999999</v>
+        <v>46.843845600000002</v>
       </c>
       <c r="L47" s="12">
         <f t="shared" si="70"/>
-        <v>43.274397280000002</v>
+        <v>44.319836850000009</v>
       </c>
       <c r="M47" s="55">
         <f t="shared" si="70"/>
-        <v>45.096966399999999</v>
+        <v>40.044045060000002</v>
       </c>
       <c r="N47" s="55">
         <f t="shared" si="70"/>
-        <v>45.3656346</v>
+        <v>44.557320990000001</v>
       </c>
       <c r="O47" s="12">
         <f t="shared" si="70"/>
-        <v>13.684520319999999</v>
+        <v>19.799229759999996</v>
       </c>
       <c r="P47" s="55">
         <f t="shared" si="70"/>
-        <v>31.163644010000002</v>
+        <v>43.161821159999995</v>
       </c>
       <c r="Q47" s="55">
         <f t="shared" si="70"/>
-        <v>31.321112970000009</v>
+        <v>29.333454150000001</v>
       </c>
       <c r="R47" s="12">
         <f t="shared" si="70"/>
-        <v>26.8180002</v>
+        <v>46.283195800000001</v>
       </c>
       <c r="S47" s="55">
         <f t="shared" si="70"/>
-        <v>32.005554619999991</v>
+        <v>44.141762300000003</v>
       </c>
       <c r="T47" s="55">
         <f t="shared" si="70"/>
-        <v>36.647047260000001</v>
+        <v>16.468300760000005</v>
       </c>
       <c r="U47" s="12">
         <f t="shared" si="70"/>
-        <v>72.64797707999999</v>
+        <v>38.112710659999998</v>
       </c>
       <c r="V47" s="55">
         <f t="shared" si="70"/>
-        <v>41.358100319999998</v>
+        <v>59.597527020000008</v>
       </c>
       <c r="W47" s="55">
         <f t="shared" si="70"/>
-        <v>54.165303640000005</v>
+        <v>33.205194159999998</v>
       </c>
       <c r="X47" s="12">
         <f t="shared" si="70"/>
-        <v>47.972380279999996</v>
+        <v>58.016290079999997</v>
       </c>
       <c r="Y47" s="55">
         <f t="shared" si="70"/>
-        <v>11.527274219999995</v>
+        <v>20.917185599999993</v>
       </c>
       <c r="Z47" s="55">
         <f t="shared" si="70"/>
-        <v>10.041190879999997</v>
+        <v>18.67922295</v>
       </c>
       <c r="AA47" s="55" t="e">
         <f t="shared" si="70"/>
@@ -17919,99 +17919,99 @@
       </c>
       <c r="C48" s="75">
         <f t="shared" ref="C48:AH48" si="75">C36*C47/100*C24/10^6</f>
-        <v>7.4807258826080844E-2</v>
+        <v>2.6026671818968457E-2</v>
       </c>
       <c r="D48" s="55">
         <f t="shared" si="75"/>
-        <v>8.1283121631102601E-2</v>
+        <v>8.3297739061776579E-2</v>
       </c>
       <c r="E48" s="13">
         <f t="shared" si="75"/>
-        <v>4.4886326674109127E-2</v>
+        <v>7.1262460760833257E-2</v>
       </c>
       <c r="F48" s="12">
         <f t="shared" si="75"/>
-        <v>8.574146819804028E-2</v>
+        <v>3.7186276682644653E-2</v>
       </c>
       <c r="G48" s="55">
         <f t="shared" si="75"/>
-        <v>8.6471430898621152E-2</v>
+        <v>3.9900143888679095E-2</v>
       </c>
       <c r="H48" s="55">
         <f t="shared" si="75"/>
-        <v>7.3445001581689789E-2</v>
+        <v>8.8461558149836958E-2</v>
       </c>
       <c r="I48" s="12">
         <f t="shared" si="75"/>
-        <v>4.7287148603355915E-2</v>
+        <v>0.11736319019443804</v>
       </c>
       <c r="J48" s="55">
         <f t="shared" si="75"/>
-        <v>3.7533892529419494E-2</v>
+        <v>4.5310435056197758E-2</v>
       </c>
       <c r="K48" s="55">
         <f t="shared" si="75"/>
-        <v>2.9988107536516036E-2</v>
+        <v>8.9575319655864225E-2</v>
       </c>
       <c r="L48" s="12">
         <f t="shared" si="75"/>
-        <v>9.1713543115002863E-2</v>
+        <v>6.5086425888374336E-2</v>
       </c>
       <c r="M48" s="55">
         <f t="shared" si="75"/>
-        <v>7.6081409551602724E-2</v>
+        <v>4.9505661897294044E-2</v>
       </c>
       <c r="N48" s="55">
         <f t="shared" si="75"/>
-        <v>3.5708772778366205E-2</v>
+        <v>6.9444460529237959E-2</v>
       </c>
       <c r="O48" s="12">
         <f t="shared" si="75"/>
-        <v>3.57998535350156E-3</v>
+        <v>3.9315673125623228E-3</v>
       </c>
       <c r="P48" s="55">
         <f t="shared" si="75"/>
-        <v>7.2692225494965026E-3</v>
+        <v>2.1532911842232473E-2</v>
       </c>
       <c r="Q48" s="55">
         <f t="shared" si="75"/>
-        <v>1.2546828849553812E-2</v>
+        <v>5.9808585905033193E-3</v>
       </c>
       <c r="R48" s="12">
         <f t="shared" si="75"/>
-        <v>4.8412204191185249E-3</v>
+        <v>3.4742687976623228E-2</v>
       </c>
       <c r="S48" s="55">
         <f t="shared" si="75"/>
-        <v>1.6596034717521337E-2</v>
+        <v>1.9895452576302475E-2</v>
       </c>
       <c r="T48" s="55">
         <f t="shared" si="75"/>
-        <v>2.294944013395471E-2</v>
+        <v>3.6232620972468208E-3</v>
       </c>
       <c r="U48" s="12">
         <f t="shared" si="75"/>
-        <v>7.6933417254571243E-2</v>
+        <v>4.1276113042328116E-2</v>
       </c>
       <c r="V48" s="55">
         <f t="shared" si="75"/>
-        <v>6.9412361138067438E-2</v>
+        <v>6.6261957755703774E-2</v>
       </c>
       <c r="W48" s="55">
         <f t="shared" si="75"/>
-        <v>0.13859108208200688</v>
+        <v>4.4368657643060097E-2</v>
       </c>
       <c r="X48" s="12">
         <f t="shared" si="75"/>
-        <v>8.0512172359702885E-2</v>
+        <v>0.16621266656166458</v>
       </c>
       <c r="Y48" s="55">
         <f t="shared" si="75"/>
-        <v>1.1649919168776175E-2</v>
+        <v>1.2753497117393675E-2</v>
       </c>
       <c r="Z48" s="55">
         <f t="shared" si="75"/>
-        <v>1.1427765557455314E-2</v>
+        <v>1.619082095731425E-2</v>
       </c>
       <c r="AA48" s="55" t="e">
         <f t="shared" si="75"/>
@@ -18573,99 +18573,99 @@
       </c>
       <c r="C50" s="75">
         <f t="shared" ref="C50:AH50" si="80">(100-C11)/(C19+1)</f>
-        <v>1.9396274599999999</v>
+        <v>0.42210009999999998</v>
       </c>
       <c r="D50" s="55">
         <f t="shared" si="80"/>
-        <v>0.40681329999999999</v>
+        <v>1.3185183</v>
       </c>
       <c r="E50" s="13">
         <f t="shared" si="80"/>
-        <v>0.43116589999999999</v>
+        <v>0.30661853999999999</v>
       </c>
       <c r="F50" s="12">
         <f t="shared" si="80"/>
-        <v>0.35360178000000003</v>
+        <v>1.3677816</v>
       </c>
       <c r="G50" s="55">
         <f t="shared" si="80"/>
-        <v>0.63618852000000004</v>
+        <v>0.51374309000000007</v>
       </c>
       <c r="H50" s="55">
         <f t="shared" si="80"/>
-        <v>1.8258913199999998</v>
+        <v>1.5946372800000002</v>
       </c>
       <c r="I50" s="12">
         <f t="shared" si="80"/>
-        <v>1.8490544799999997</v>
+        <v>0.33238463999999995</v>
       </c>
       <c r="J50" s="55">
         <f t="shared" si="80"/>
-        <v>1.44131247</v>
+        <v>1.88211624</v>
       </c>
       <c r="K50" s="55">
         <f t="shared" si="80"/>
-        <v>1.45160208</v>
+        <v>1.0121544000000002</v>
       </c>
       <c r="L50" s="12">
         <f t="shared" si="80"/>
-        <v>1.9936027199999997</v>
+        <v>1.6851631499999997</v>
       </c>
       <c r="M50" s="55">
         <f t="shared" si="80"/>
-        <v>0.39303359999999998</v>
+        <v>1.4549549400000001</v>
       </c>
       <c r="N50" s="55">
         <f t="shared" si="80"/>
-        <v>1.4943654000000002</v>
+        <v>1.59167901</v>
       </c>
       <c r="O50" s="12">
         <f t="shared" si="80"/>
-        <v>3.0234796799999999</v>
+        <v>2.1287702399999997</v>
       </c>
       <c r="P50" s="55">
         <f t="shared" si="80"/>
-        <v>3.6673559900000003</v>
+        <v>5.0001788400000002</v>
       </c>
       <c r="Q50" s="55">
         <f t="shared" si="80"/>
-        <v>3.6858870300000004</v>
+        <v>7.2615458499999992</v>
       </c>
       <c r="R50" s="12">
         <f t="shared" si="80"/>
-        <v>6.2269998000000015</v>
+        <v>1.8808042</v>
       </c>
       <c r="S50" s="55">
         <f t="shared" si="80"/>
-        <v>2.8084453799999998</v>
+        <v>4.0132376999999995</v>
       </c>
       <c r="T50" s="55">
         <f t="shared" si="80"/>
-        <v>1.2639527400000001</v>
+        <v>3.6576992400000008</v>
       </c>
       <c r="U50" s="12">
         <f t="shared" si="80"/>
-        <v>0.39002292</v>
+        <v>6.0902893400000018</v>
       </c>
       <c r="V50" s="55">
         <f t="shared" si="80"/>
-        <v>8.5478996799999987</v>
+        <v>5.9684729799999996</v>
       </c>
       <c r="W50" s="55">
         <f t="shared" si="80"/>
-        <v>9.657696360000001</v>
+        <v>7.34680584</v>
       </c>
       <c r="X50" s="12">
         <f t="shared" si="80"/>
-        <v>9.065619719999999</v>
+        <v>2.5157099199999999</v>
       </c>
       <c r="Y50" s="55">
         <f t="shared" si="80"/>
-        <v>0.71572577999999965</v>
+        <v>1.6618143999999995</v>
       </c>
       <c r="Z50" s="55">
         <f t="shared" si="80"/>
-        <v>0.65480911999999991</v>
+        <v>2.6657770499999995</v>
       </c>
       <c r="AA50" s="55" t="e">
         <f t="shared" si="80"/>
@@ -19133,99 +19133,99 @@
       </c>
       <c r="C51" s="75">
         <f t="shared" ref="C51:AH51" si="85">C36*C50/100*C25/10^6</f>
-        <v>2.0080012264491905E-2</v>
+        <v>1.4888854741902835E-3</v>
       </c>
       <c r="D51" s="55">
         <f t="shared" si="85"/>
-        <v>4.746192457512924E-3</v>
+        <v>1.5543172123046949E-2</v>
       </c>
       <c r="E51" s="13">
         <f t="shared" si="85"/>
-        <v>2.7391948983270229E-3</v>
+        <v>3.0705833709740514E-3</v>
       </c>
       <c r="F51" s="12">
         <f t="shared" si="85"/>
-        <v>4.4595483876663268E-3</v>
+        <v>7.8970018414403018E-3</v>
       </c>
       <c r="G51" s="55">
         <f t="shared" si="85"/>
-        <v>7.6051950267521009E-3</v>
+        <v>2.9247820596998405E-3</v>
       </c>
       <c r="H51" s="55">
         <f t="shared" si="85"/>
-        <v>2.0260984123611839E-2</v>
+        <v>2.0536212155800863E-2</v>
       </c>
       <c r="I51" s="12">
         <f t="shared" si="85"/>
-        <v>1.2712873869823586E-2</v>
+        <v>4.4883624700036802E-3</v>
       </c>
       <c r="J51" s="55">
         <f t="shared" si="85"/>
-        <v>7.7716377978469106E-3</v>
+        <v>1.2028961699535186E-2</v>
       </c>
       <c r="K51" s="55">
         <f t="shared" si="85"/>
-        <v>7.0407892873508258E-3</v>
+        <v>1.251411364068733E-2</v>
       </c>
       <c r="L51" s="12">
         <f t="shared" si="85"/>
-        <v>2.7318607761455824E-2</v>
+        <v>1.600116949726826E-2</v>
       </c>
       <c r="M51" s="55">
         <f t="shared" si="85"/>
-        <v>4.2872459834892677E-3</v>
+        <v>1.1630114080400336E-2</v>
       </c>
       <c r="N51" s="55">
         <f t="shared" si="85"/>
-        <v>7.6054031319156947E-3</v>
+        <v>1.6039525928285919E-2</v>
       </c>
       <c r="O51" s="12">
         <f t="shared" si="85"/>
-        <v>5.1141825555395468E-3</v>
+        <v>2.7331515387334759E-3</v>
       </c>
       <c r="P51" s="55">
         <f t="shared" si="85"/>
-        <v>5.5310845933975528E-3</v>
+        <v>1.6128947958707895E-2</v>
       </c>
       <c r="Q51" s="55">
         <f t="shared" si="85"/>
-        <v>9.5467666966077142E-3</v>
+        <v>9.5729747454755126E-3</v>
       </c>
       <c r="R51" s="12">
         <f t="shared" si="85"/>
-        <v>7.2681656989022504E-3</v>
+        <v>9.1285366669399647E-3</v>
       </c>
       <c r="S51" s="55">
         <f t="shared" si="85"/>
-        <v>9.4159135059521965E-3</v>
+        <v>1.169543930945607E-2</v>
       </c>
       <c r="T51" s="55">
         <f t="shared" si="85"/>
-        <v>5.1177780095669123E-3</v>
+        <v>5.2032711038009884E-3</v>
       </c>
       <c r="U51" s="12">
         <f t="shared" si="85"/>
-        <v>2.670540253634745E-3</v>
+        <v>4.2646597016949839E-2</v>
       </c>
       <c r="V51" s="55">
         <f t="shared" si="85"/>
-        <v>9.2758379567373303E-2</v>
+        <v>4.2905874434766511E-2</v>
       </c>
       <c r="W51" s="55">
         <f t="shared" si="85"/>
-        <v>0.15977364821461151</v>
+        <v>6.3472605965280579E-2</v>
       </c>
       <c r="X51" s="12">
         <f t="shared" si="85"/>
-        <v>9.837512018676968E-2</v>
+        <v>4.6600677067801757E-2</v>
       </c>
       <c r="Y51" s="55">
         <f t="shared" si="85"/>
-        <v>4.6769254708000493E-3</v>
+        <v>6.5512784329832948E-3</v>
       </c>
       <c r="Z51" s="55">
         <f t="shared" si="85"/>
-        <v>4.8184606871808644E-3</v>
+        <v>1.4940027281839994E-2</v>
       </c>
       <c r="AA51" s="55" t="e">
         <f t="shared" si="85"/>
@@ -19929,66 +19929,110 @@
       <c r="B54" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="C54" s="79"/>
-      <c r="D54" s="59"/>
-      <c r="E54" s="30"/>
-      <c r="F54" s="31"/>
-      <c r="G54" s="59"/>
-      <c r="H54" s="59"/>
-      <c r="I54" s="31"/>
-      <c r="J54" s="59"/>
-      <c r="K54" s="59"/>
-      <c r="L54" s="31"/>
-      <c r="M54" s="59"/>
-      <c r="N54" s="59"/>
-      <c r="O54" s="31"/>
-      <c r="P54" s="59"/>
-      <c r="Q54" s="59"/>
-      <c r="R54" s="31"/>
-      <c r="S54" s="59"/>
-      <c r="T54" s="59"/>
-      <c r="U54" s="31"/>
-      <c r="V54" s="59"/>
-      <c r="W54" s="59"/>
-      <c r="X54" s="31"/>
-      <c r="Y54" s="59"/>
-      <c r="Z54" s="59"/>
-      <c r="AA54" s="59"/>
-      <c r="AB54" s="31"/>
-      <c r="AC54" s="59"/>
-      <c r="AD54" s="59"/>
-      <c r="AE54" s="31"/>
-      <c r="AF54" s="59"/>
-      <c r="AG54" s="59"/>
-      <c r="AH54" s="31"/>
-      <c r="AI54" s="59"/>
-      <c r="AJ54" s="59"/>
-      <c r="AK54" s="31"/>
-      <c r="AL54" s="59"/>
-      <c r="AM54" s="59"/>
-      <c r="AN54" s="31"/>
-      <c r="AO54" s="59"/>
-      <c r="AP54" s="59"/>
-      <c r="AQ54" s="31"/>
-      <c r="AR54" s="59"/>
-      <c r="AS54" s="59"/>
-      <c r="AT54" s="59"/>
-      <c r="AU54" s="31"/>
-      <c r="AV54" s="59"/>
-      <c r="AW54" s="59"/>
-      <c r="AX54" s="31"/>
-      <c r="AY54" s="59"/>
-      <c r="AZ54" s="59"/>
-      <c r="BA54" s="31"/>
-      <c r="BB54" s="59"/>
-      <c r="BC54" s="59"/>
-      <c r="BD54" s="31"/>
-      <c r="BE54" s="59"/>
-      <c r="BF54" s="59"/>
-      <c r="BG54" s="31"/>
-      <c r="BH54" s="59"/>
-      <c r="BI54" s="59"/>
-      <c r="BJ54" s="31"/>
+      <c r="C54" s="79">
+        <v>15</v>
+      </c>
+      <c r="D54" s="79">
+        <v>15</v>
+      </c>
+      <c r="E54" s="79">
+        <v>15</v>
+      </c>
+      <c r="F54" s="79">
+        <v>15</v>
+      </c>
+      <c r="G54" s="79">
+        <v>15</v>
+      </c>
+      <c r="H54" s="79">
+        <v>15</v>
+      </c>
+      <c r="I54" s="79">
+        <v>15</v>
+      </c>
+      <c r="J54" s="79">
+        <v>15</v>
+      </c>
+      <c r="K54" s="79">
+        <v>15</v>
+      </c>
+      <c r="L54" s="79">
+        <v>15</v>
+      </c>
+      <c r="M54" s="79">
+        <v>15</v>
+      </c>
+      <c r="N54" s="79">
+        <v>15</v>
+      </c>
+      <c r="O54" s="79">
+        <v>15</v>
+      </c>
+      <c r="P54" s="79">
+        <v>5</v>
+      </c>
+      <c r="Q54" s="79">
+        <v>15</v>
+      </c>
+      <c r="R54" s="79">
+        <v>5</v>
+      </c>
+      <c r="S54" s="79">
+        <v>15</v>
+      </c>
+      <c r="T54" s="79">
+        <v>15</v>
+      </c>
+      <c r="U54" s="79">
+        <v>15</v>
+      </c>
+      <c r="V54" s="79">
+        <v>15</v>
+      </c>
+      <c r="W54" s="79">
+        <v>15</v>
+      </c>
+      <c r="X54" s="79">
+        <v>15</v>
+      </c>
+      <c r="Y54" s="79"/>
+      <c r="Z54" s="79"/>
+      <c r="AA54" s="79"/>
+      <c r="AB54" s="79"/>
+      <c r="AC54" s="79"/>
+      <c r="AD54" s="79"/>
+      <c r="AE54" s="79"/>
+      <c r="AF54" s="79"/>
+      <c r="AG54" s="79"/>
+      <c r="AH54" s="79"/>
+      <c r="AI54" s="79"/>
+      <c r="AJ54" s="79"/>
+      <c r="AK54" s="79"/>
+      <c r="AL54" s="79"/>
+      <c r="AM54" s="79"/>
+      <c r="AN54" s="79"/>
+      <c r="AO54" s="79"/>
+      <c r="AP54" s="79"/>
+      <c r="AQ54" s="79"/>
+      <c r="AR54" s="79"/>
+      <c r="AS54" s="79"/>
+      <c r="AT54" s="79"/>
+      <c r="AU54" s="79"/>
+      <c r="AV54" s="79"/>
+      <c r="AW54" s="79"/>
+      <c r="AX54" s="79"/>
+      <c r="AY54" s="79"/>
+      <c r="AZ54" s="79"/>
+      <c r="BA54" s="79"/>
+      <c r="BB54" s="79"/>
+      <c r="BC54" s="79"/>
+      <c r="BD54" s="79"/>
+      <c r="BE54" s="79"/>
+      <c r="BF54" s="79"/>
+      <c r="BG54" s="79"/>
+      <c r="BH54" s="79"/>
+      <c r="BI54" s="79"/>
+      <c r="BJ54" s="79"/>
       <c r="BK54" s="59"/>
       <c r="BL54" s="59"/>
       <c r="BM54" s="59"/>
@@ -20075,66 +20119,110 @@
       <c r="B55" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="C55" s="80"/>
-      <c r="D55" s="60"/>
-      <c r="E55" s="32"/>
-      <c r="F55" s="33"/>
-      <c r="G55" s="60"/>
-      <c r="H55" s="60"/>
-      <c r="I55" s="33"/>
-      <c r="J55" s="60"/>
-      <c r="K55" s="60"/>
-      <c r="L55" s="33"/>
-      <c r="M55" s="60"/>
-      <c r="N55" s="60"/>
-      <c r="O55" s="33"/>
-      <c r="P55" s="60"/>
-      <c r="Q55" s="60"/>
-      <c r="R55" s="33"/>
-      <c r="S55" s="60"/>
-      <c r="T55" s="60"/>
-      <c r="U55" s="33"/>
-      <c r="V55" s="60"/>
-      <c r="W55" s="60"/>
-      <c r="X55" s="33"/>
-      <c r="Y55" s="60"/>
-      <c r="Z55" s="60"/>
-      <c r="AA55" s="60"/>
-      <c r="AB55" s="33"/>
-      <c r="AC55" s="60"/>
-      <c r="AD55" s="60"/>
-      <c r="AE55" s="33"/>
-      <c r="AF55" s="60"/>
-      <c r="AG55" s="60"/>
-      <c r="AH55" s="33"/>
-      <c r="AI55" s="60"/>
-      <c r="AJ55" s="60"/>
-      <c r="AK55" s="33"/>
-      <c r="AL55" s="60"/>
-      <c r="AM55" s="60"/>
-      <c r="AN55" s="33"/>
-      <c r="AO55" s="60"/>
-      <c r="AP55" s="60"/>
-      <c r="AQ55" s="33"/>
-      <c r="AR55" s="60"/>
-      <c r="AS55" s="60"/>
-      <c r="AT55" s="60"/>
-      <c r="AU55" s="33"/>
-      <c r="AV55" s="60"/>
-      <c r="AW55" s="60"/>
-      <c r="AX55" s="33"/>
-      <c r="AY55" s="60"/>
-      <c r="AZ55" s="60"/>
-      <c r="BA55" s="33"/>
-      <c r="BB55" s="60"/>
-      <c r="BC55" s="60"/>
-      <c r="BD55" s="33"/>
-      <c r="BE55" s="60"/>
-      <c r="BF55" s="60"/>
-      <c r="BG55" s="33"/>
-      <c r="BH55" s="60"/>
-      <c r="BI55" s="60"/>
-      <c r="BJ55" s="33"/>
+      <c r="C55" s="80">
+        <v>5</v>
+      </c>
+      <c r="D55" s="80">
+        <v>5</v>
+      </c>
+      <c r="E55" s="80">
+        <v>5</v>
+      </c>
+      <c r="F55" s="80">
+        <v>5</v>
+      </c>
+      <c r="G55" s="80">
+        <v>5</v>
+      </c>
+      <c r="H55" s="80">
+        <v>5</v>
+      </c>
+      <c r="I55" s="80">
+        <v>5</v>
+      </c>
+      <c r="J55" s="80">
+        <v>5</v>
+      </c>
+      <c r="K55" s="80">
+        <v>5</v>
+      </c>
+      <c r="L55" s="80">
+        <v>5</v>
+      </c>
+      <c r="M55" s="80">
+        <v>5</v>
+      </c>
+      <c r="N55" s="80">
+        <v>5</v>
+      </c>
+      <c r="O55" s="80">
+        <v>0.01</v>
+      </c>
+      <c r="P55" s="80">
+        <v>5</v>
+      </c>
+      <c r="Q55" s="80">
+        <v>0.01</v>
+      </c>
+      <c r="R55" s="80">
+        <v>5</v>
+      </c>
+      <c r="S55" s="80">
+        <v>5</v>
+      </c>
+      <c r="T55" s="80">
+        <v>0.1</v>
+      </c>
+      <c r="U55" s="80">
+        <v>5</v>
+      </c>
+      <c r="V55" s="80">
+        <v>5</v>
+      </c>
+      <c r="W55" s="80">
+        <v>5</v>
+      </c>
+      <c r="X55" s="80">
+        <v>5</v>
+      </c>
+      <c r="Y55" s="80"/>
+      <c r="Z55" s="80"/>
+      <c r="AA55" s="80"/>
+      <c r="AB55" s="80"/>
+      <c r="AC55" s="80"/>
+      <c r="AD55" s="80"/>
+      <c r="AE55" s="80"/>
+      <c r="AF55" s="80"/>
+      <c r="AG55" s="80"/>
+      <c r="AH55" s="80"/>
+      <c r="AI55" s="80"/>
+      <c r="AJ55" s="80"/>
+      <c r="AK55" s="80"/>
+      <c r="AL55" s="80"/>
+      <c r="AM55" s="80"/>
+      <c r="AN55" s="80"/>
+      <c r="AO55" s="80"/>
+      <c r="AP55" s="80"/>
+      <c r="AQ55" s="80"/>
+      <c r="AR55" s="80"/>
+      <c r="AS55" s="80"/>
+      <c r="AT55" s="80"/>
+      <c r="AU55" s="80"/>
+      <c r="AV55" s="80"/>
+      <c r="AW55" s="80"/>
+      <c r="AX55" s="80"/>
+      <c r="AY55" s="80"/>
+      <c r="AZ55" s="80"/>
+      <c r="BA55" s="80"/>
+      <c r="BB55" s="80"/>
+      <c r="BC55" s="80"/>
+      <c r="BD55" s="80"/>
+      <c r="BE55" s="80"/>
+      <c r="BF55" s="80"/>
+      <c r="BG55" s="80"/>
+      <c r="BH55" s="80"/>
+      <c r="BI55" s="80"/>
+      <c r="BJ55" s="80"/>
       <c r="BK55" s="60"/>
       <c r="BL55" s="60"/>
       <c r="BM55" s="60"/>
@@ -20221,66 +20309,110 @@
       <c r="B56" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="C56" s="80"/>
-      <c r="D56" s="60"/>
-      <c r="E56" s="32"/>
-      <c r="F56" s="33"/>
-      <c r="G56" s="60"/>
-      <c r="H56" s="60"/>
-      <c r="I56" s="33"/>
-      <c r="J56" s="60"/>
-      <c r="K56" s="60"/>
-      <c r="L56" s="33"/>
-      <c r="M56" s="60"/>
-      <c r="N56" s="60"/>
-      <c r="O56" s="33"/>
-      <c r="P56" s="60"/>
-      <c r="Q56" s="60"/>
-      <c r="R56" s="33"/>
-      <c r="S56" s="60"/>
-      <c r="T56" s="60"/>
-      <c r="U56" s="33"/>
-      <c r="V56" s="60"/>
-      <c r="W56" s="60"/>
-      <c r="X56" s="33"/>
-      <c r="Y56" s="60"/>
-      <c r="Z56" s="60"/>
-      <c r="AA56" s="60"/>
-      <c r="AB56" s="33"/>
-      <c r="AC56" s="60"/>
-      <c r="AD56" s="60"/>
-      <c r="AE56" s="33"/>
-      <c r="AF56" s="60"/>
-      <c r="AG56" s="60"/>
-      <c r="AH56" s="33"/>
-      <c r="AI56" s="60"/>
-      <c r="AJ56" s="60"/>
-      <c r="AK56" s="33"/>
-      <c r="AL56" s="60"/>
-      <c r="AM56" s="60"/>
-      <c r="AN56" s="33"/>
-      <c r="AO56" s="60"/>
-      <c r="AP56" s="60"/>
-      <c r="AQ56" s="33"/>
-      <c r="AR56" s="60"/>
-      <c r="AS56" s="60"/>
-      <c r="AT56" s="60"/>
-      <c r="AU56" s="33"/>
-      <c r="AV56" s="60"/>
-      <c r="AW56" s="60"/>
-      <c r="AX56" s="33"/>
-      <c r="AY56" s="60"/>
-      <c r="AZ56" s="60"/>
-      <c r="BA56" s="33"/>
-      <c r="BB56" s="60"/>
-      <c r="BC56" s="60"/>
-      <c r="BD56" s="33"/>
-      <c r="BE56" s="60"/>
-      <c r="BF56" s="60"/>
-      <c r="BG56" s="33"/>
-      <c r="BH56" s="60"/>
-      <c r="BI56" s="60"/>
-      <c r="BJ56" s="33"/>
+      <c r="C56" s="80">
+        <v>5</v>
+      </c>
+      <c r="D56" s="80">
+        <v>5</v>
+      </c>
+      <c r="E56" s="80">
+        <v>5</v>
+      </c>
+      <c r="F56" s="80">
+        <v>5</v>
+      </c>
+      <c r="G56" s="80">
+        <v>5</v>
+      </c>
+      <c r="H56" s="80">
+        <v>5</v>
+      </c>
+      <c r="I56" s="80">
+        <v>5</v>
+      </c>
+      <c r="J56" s="80">
+        <v>5</v>
+      </c>
+      <c r="K56" s="80">
+        <v>5</v>
+      </c>
+      <c r="L56" s="80">
+        <v>5</v>
+      </c>
+      <c r="M56" s="80">
+        <v>5</v>
+      </c>
+      <c r="N56" s="80">
+        <v>5</v>
+      </c>
+      <c r="O56" s="80">
+        <v>1</v>
+      </c>
+      <c r="P56" s="80">
+        <v>5</v>
+      </c>
+      <c r="Q56" s="80">
+        <v>1</v>
+      </c>
+      <c r="R56" s="80">
+        <v>5</v>
+      </c>
+      <c r="S56" s="80">
+        <v>5</v>
+      </c>
+      <c r="T56" s="80">
+        <v>1</v>
+      </c>
+      <c r="U56" s="80">
+        <v>5</v>
+      </c>
+      <c r="V56" s="80">
+        <v>5</v>
+      </c>
+      <c r="W56" s="80">
+        <v>5</v>
+      </c>
+      <c r="X56" s="80">
+        <v>15</v>
+      </c>
+      <c r="Y56" s="80"/>
+      <c r="Z56" s="80"/>
+      <c r="AA56" s="80"/>
+      <c r="AB56" s="80"/>
+      <c r="AC56" s="80"/>
+      <c r="AD56" s="80"/>
+      <c r="AE56" s="80"/>
+      <c r="AF56" s="80"/>
+      <c r="AG56" s="80"/>
+      <c r="AH56" s="80"/>
+      <c r="AI56" s="80"/>
+      <c r="AJ56" s="80"/>
+      <c r="AK56" s="80"/>
+      <c r="AL56" s="80"/>
+      <c r="AM56" s="80"/>
+      <c r="AN56" s="80"/>
+      <c r="AO56" s="80"/>
+      <c r="AP56" s="80"/>
+      <c r="AQ56" s="80"/>
+      <c r="AR56" s="80"/>
+      <c r="AS56" s="80"/>
+      <c r="AT56" s="80"/>
+      <c r="AU56" s="80"/>
+      <c r="AV56" s="80"/>
+      <c r="AW56" s="80"/>
+      <c r="AX56" s="80"/>
+      <c r="AY56" s="80"/>
+      <c r="AZ56" s="80"/>
+      <c r="BA56" s="80"/>
+      <c r="BB56" s="80"/>
+      <c r="BC56" s="80"/>
+      <c r="BD56" s="80"/>
+      <c r="BE56" s="80"/>
+      <c r="BF56" s="80"/>
+      <c r="BG56" s="80"/>
+      <c r="BH56" s="80"/>
+      <c r="BI56" s="80"/>
+      <c r="BJ56" s="80"/>
       <c r="BK56" s="60"/>
       <c r="BL56" s="60"/>
       <c r="BM56" s="60"/>
@@ -20367,66 +20499,110 @@
       <c r="B57" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="C57" s="81"/>
-      <c r="D57" s="61"/>
-      <c r="E57" s="34"/>
-      <c r="F57" s="35"/>
-      <c r="G57" s="61"/>
-      <c r="H57" s="61"/>
-      <c r="I57" s="35"/>
-      <c r="J57" s="61"/>
-      <c r="K57" s="61"/>
-      <c r="L57" s="35"/>
-      <c r="M57" s="61"/>
-      <c r="N57" s="61"/>
-      <c r="O57" s="35"/>
-      <c r="P57" s="61"/>
-      <c r="Q57" s="61"/>
-      <c r="R57" s="35"/>
-      <c r="S57" s="61"/>
-      <c r="T57" s="61"/>
-      <c r="U57" s="35"/>
-      <c r="V57" s="61"/>
-      <c r="W57" s="61"/>
-      <c r="X57" s="35"/>
-      <c r="Y57" s="61"/>
-      <c r="Z57" s="61"/>
-      <c r="AA57" s="61"/>
-      <c r="AB57" s="35"/>
-      <c r="AC57" s="61"/>
-      <c r="AD57" s="61"/>
-      <c r="AE57" s="35"/>
-      <c r="AF57" s="61"/>
-      <c r="AG57" s="61"/>
-      <c r="AH57" s="35"/>
-      <c r="AI57" s="61"/>
-      <c r="AJ57" s="61"/>
-      <c r="AK57" s="35"/>
-      <c r="AL57" s="61"/>
-      <c r="AM57" s="61"/>
-      <c r="AN57" s="35"/>
-      <c r="AO57" s="61"/>
-      <c r="AP57" s="61"/>
-      <c r="AQ57" s="35"/>
-      <c r="AR57" s="61"/>
-      <c r="AS57" s="61"/>
-      <c r="AT57" s="61"/>
-      <c r="AU57" s="35"/>
-      <c r="AV57" s="61"/>
-      <c r="AW57" s="61"/>
-      <c r="AX57" s="35"/>
-      <c r="AY57" s="61"/>
-      <c r="AZ57" s="61"/>
-      <c r="BA57" s="35"/>
-      <c r="BB57" s="61"/>
-      <c r="BC57" s="61"/>
-      <c r="BD57" s="35"/>
-      <c r="BE57" s="61"/>
-      <c r="BF57" s="61"/>
-      <c r="BG57" s="35"/>
-      <c r="BH57" s="61"/>
-      <c r="BI57" s="61"/>
-      <c r="BJ57" s="35"/>
+      <c r="C57" s="81">
+        <v>1</v>
+      </c>
+      <c r="D57" s="81">
+        <v>5</v>
+      </c>
+      <c r="E57" s="81">
+        <v>1</v>
+      </c>
+      <c r="F57" s="81">
+        <v>1</v>
+      </c>
+      <c r="G57" s="81">
+        <v>1</v>
+      </c>
+      <c r="H57" s="81">
+        <v>5</v>
+      </c>
+      <c r="I57" s="81">
+        <v>1</v>
+      </c>
+      <c r="J57" s="81">
+        <v>1</v>
+      </c>
+      <c r="K57" s="81">
+        <v>5</v>
+      </c>
+      <c r="L57" s="81">
+        <v>1</v>
+      </c>
+      <c r="M57" s="81">
+        <v>1</v>
+      </c>
+      <c r="N57" s="81">
+        <v>5</v>
+      </c>
+      <c r="O57" s="81">
+        <v>1</v>
+      </c>
+      <c r="P57" s="81">
+        <v>1</v>
+      </c>
+      <c r="Q57" s="81">
+        <v>1</v>
+      </c>
+      <c r="R57" s="81">
+        <v>1</v>
+      </c>
+      <c r="S57" s="81">
+        <v>1</v>
+      </c>
+      <c r="T57" s="81">
+        <v>1</v>
+      </c>
+      <c r="U57" s="81">
+        <v>5</v>
+      </c>
+      <c r="V57" s="81">
+        <v>5</v>
+      </c>
+      <c r="W57" s="81">
+        <v>5</v>
+      </c>
+      <c r="X57" s="81">
+        <v>5</v>
+      </c>
+      <c r="Y57" s="81"/>
+      <c r="Z57" s="81"/>
+      <c r="AA57" s="81"/>
+      <c r="AB57" s="81"/>
+      <c r="AC57" s="81"/>
+      <c r="AD57" s="81"/>
+      <c r="AE57" s="81"/>
+      <c r="AF57" s="81"/>
+      <c r="AG57" s="81"/>
+      <c r="AH57" s="81"/>
+      <c r="AI57" s="81"/>
+      <c r="AJ57" s="81"/>
+      <c r="AK57" s="81"/>
+      <c r="AL57" s="81"/>
+      <c r="AM57" s="81"/>
+      <c r="AN57" s="81"/>
+      <c r="AO57" s="81"/>
+      <c r="AP57" s="81"/>
+      <c r="AQ57" s="81"/>
+      <c r="AR57" s="81"/>
+      <c r="AS57" s="81"/>
+      <c r="AT57" s="81"/>
+      <c r="AU57" s="81"/>
+      <c r="AV57" s="81"/>
+      <c r="AW57" s="81"/>
+      <c r="AX57" s="81"/>
+      <c r="AY57" s="81"/>
+      <c r="AZ57" s="81"/>
+      <c r="BA57" s="81"/>
+      <c r="BB57" s="81"/>
+      <c r="BC57" s="81"/>
+      <c r="BD57" s="81"/>
+      <c r="BE57" s="81"/>
+      <c r="BF57" s="81"/>
+      <c r="BG57" s="81"/>
+      <c r="BH57" s="81"/>
+      <c r="BI57" s="81"/>
+      <c r="BJ57" s="81"/>
       <c r="BK57" s="61"/>
       <c r="BL57" s="61"/>
       <c r="BM57" s="61"/>
@@ -21692,93 +21868,93 @@
       <c r="B63" s="93" t="s">
         <v>37</v>
       </c>
-      <c r="C63" s="82" t="e">
+      <c r="C63" s="82">
         <f t="shared" ref="C63:AH63" si="90">C42/C32</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D63" s="62" t="e">
+        <v>2.4095914587276002</v>
+      </c>
+      <c r="D63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E63" s="37" t="e">
+        <v>7.8872282453016007</v>
+      </c>
+      <c r="E63" s="37">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F63" s="47" t="e">
+        <v>7.5099010775039989</v>
+      </c>
+      <c r="F63" s="47">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G63" s="62" t="e">
+        <v>4.2171607203695984</v>
+      </c>
+      <c r="G63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H63" s="62" t="e">
+        <v>4.1922799897056002</v>
+      </c>
+      <c r="H63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I63" s="47" t="e">
+        <v>8.7967148921585991</v>
+      </c>
+      <c r="I63" s="47">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J63" s="62" t="e">
+        <v>7.7446093333986008</v>
+      </c>
+      <c r="J63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K63" s="62" t="e">
+        <v>2.8688636419740003</v>
+      </c>
+      <c r="K63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L63" s="47" t="e">
+        <v>5.1774232665455999</v>
+      </c>
+      <c r="L63" s="47">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M63" s="62" t="e">
+        <v>4.7208092331648004</v>
+      </c>
+      <c r="M63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N63" s="62" t="e">
+        <v>5.9031392992980001</v>
+      </c>
+      <c r="N63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O63" s="47" t="e">
+        <v>3.7812509625105006</v>
+      </c>
+      <c r="O63" s="47">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P63" s="62" t="e">
+        <v>1.7134060118966998</v>
+      </c>
+      <c r="P63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q63" s="62" t="e">
+        <v>1.7250625458612006</v>
+      </c>
+      <c r="Q63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R63" s="47" t="e">
+        <v>1.4304457519506</v>
+      </c>
+      <c r="R63" s="47">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S63" s="62" t="e">
+        <v>2.6247314568330009</v>
+      </c>
+      <c r="S63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T63" s="62" t="e">
+        <v>1.0591357315401002</v>
+      </c>
+      <c r="T63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U63" s="47" t="e">
+        <v>1.9341318783779999</v>
+      </c>
+      <c r="U63" s="47">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V63" s="62" t="e">
+        <v>3.9625158203901001</v>
+      </c>
+      <c r="V63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W63" s="62" t="e">
+        <v>3.6727320250676998</v>
+      </c>
+      <c r="W63" s="62">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X63" s="47" t="e">
+        <v>3.7540103135232004</v>
+      </c>
+      <c r="X63" s="47">
         <f t="shared" si="90"/>
-        <v>#DIV/0!</v>
+        <v>11.604108651547202</v>
       </c>
       <c r="Y63" s="62" t="e">
         <f t="shared" si="90"/>
@@ -22252,93 +22428,93 @@
       <c r="B64" s="94" t="s">
         <v>37</v>
       </c>
-      <c r="C64" s="83" t="e">
+      <c r="C64" s="83">
         <f t="shared" ref="C64:AH64" si="95">C45/C31</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D64" s="63" t="e">
+        <v>2.6697459399365995</v>
+      </c>
+      <c r="D64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E64" s="39" t="e">
+        <v>10.371411095295599</v>
+      </c>
+      <c r="E64" s="39">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F64" s="28" t="e">
+        <v>6.2578877168639995</v>
+      </c>
+      <c r="F64" s="28">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G64" s="63" t="e">
+        <v>5.229498575733599</v>
+      </c>
+      <c r="G64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H64" s="63" t="e">
+        <v>4.0176127338096004</v>
+      </c>
+      <c r="H64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I64" s="28" t="e">
+        <v>11.477343944720097</v>
+      </c>
+      <c r="I64" s="28">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J64" s="63" t="e">
+        <v>8.5156371200601004</v>
+      </c>
+      <c r="J64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K64" s="63" t="e">
+        <v>10.529451884259</v>
+      </c>
+      <c r="K64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L64" s="28" t="e">
+        <v>21.638772283749599</v>
+      </c>
+      <c r="L64" s="28">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M64" s="63" t="e">
+        <v>14.980545402796801</v>
+      </c>
+      <c r="M64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N64" s="63" t="e">
+        <v>7.7664169059930002</v>
+      </c>
+      <c r="N64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O64" s="28" t="e">
+        <v>20.343136105049251</v>
+      </c>
+      <c r="O64" s="28">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P64" s="63" t="e">
+        <v>5.3540659779749982</v>
+      </c>
+      <c r="P64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q64" s="63" t="e">
+        <v>8.4469371254813996</v>
+      </c>
+      <c r="Q64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R64" s="28" t="e">
+        <v>1.4265988960499998</v>
+      </c>
+      <c r="R64" s="28">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S64" s="63" t="e">
+        <v>12.673298661913499</v>
+      </c>
+      <c r="S64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T64" s="63" t="e">
+        <v>5.6404195275928499</v>
+      </c>
+      <c r="T64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U64" s="28" t="e">
+        <v>2.1044484886499997</v>
+      </c>
+      <c r="U64" s="28">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V64" s="63" t="e">
+        <v>10.06894915981785</v>
+      </c>
+      <c r="V64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W64" s="63" t="e">
+        <v>2.0884373143294503</v>
+      </c>
+      <c r="W64" s="63">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X64" s="28" t="e">
+        <v>18.606614613811196</v>
+      </c>
+      <c r="X64" s="28">
         <f t="shared" si="95"/>
-        <v>#DIV/0!</v>
+        <v>3.3745463354951997</v>
       </c>
       <c r="Y64" s="63" t="e">
         <f t="shared" si="95"/>
@@ -22812,93 +22988,93 @@
       <c r="B65" s="94" t="s">
         <v>37</v>
       </c>
-      <c r="C65" s="83" t="e">
+      <c r="C65" s="83">
         <f t="shared" ref="C65:AH65" si="100">C48/C56*1000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D65" s="63" t="e">
+        <v>5.2053343637936909</v>
+      </c>
+      <c r="D65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E65" s="39" t="e">
+        <v>16.659547812355314</v>
+      </c>
+      <c r="E65" s="39">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F65" s="28" t="e">
+        <v>14.252492152166651</v>
+      </c>
+      <c r="F65" s="28">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G65" s="63" t="e">
+        <v>7.4372553365289304</v>
+      </c>
+      <c r="G65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H65" s="63" t="e">
+        <v>7.9800287777358188</v>
+      </c>
+      <c r="H65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I65" s="28" t="e">
+        <v>17.692311629967392</v>
+      </c>
+      <c r="I65" s="28">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J65" s="63" t="e">
+        <v>23.472638038887609</v>
+      </c>
+      <c r="J65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K65" s="63" t="e">
+        <v>9.0620870112395515</v>
+      </c>
+      <c r="K65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L65" s="28" t="e">
+        <v>17.915063931172845</v>
+      </c>
+      <c r="L65" s="28">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M65" s="63" t="e">
+        <v>13.017285177674868</v>
+      </c>
+      <c r="M65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N65" s="63" t="e">
+        <v>9.901132379458808</v>
+      </c>
+      <c r="N65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O65" s="28" t="e">
+        <v>13.88889210584759</v>
+      </c>
+      <c r="O65" s="28">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P65" s="63" t="e">
+        <v>3.9315673125623229</v>
+      </c>
+      <c r="P65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q65" s="63" t="e">
+        <v>4.3065823684464943</v>
+      </c>
+      <c r="Q65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R65" s="28" t="e">
+        <v>5.9808585905033196</v>
+      </c>
+      <c r="R65" s="28">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S65" s="63" t="e">
+        <v>6.9485375953246455</v>
+      </c>
+      <c r="S65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T65" s="63" t="e">
+        <v>3.979090515260495</v>
+      </c>
+      <c r="T65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U65" s="28" t="e">
+        <v>3.6232620972468208</v>
+      </c>
+      <c r="U65" s="28">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V65" s="63" t="e">
+        <v>8.2552226084656226</v>
+      </c>
+      <c r="V65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W65" s="63" t="e">
+        <v>13.252391551140756</v>
+      </c>
+      <c r="W65" s="63">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X65" s="28" t="e">
+        <v>8.8737315286120193</v>
+      </c>
+      <c r="X65" s="28">
         <f t="shared" si="100"/>
-        <v>#DIV/0!</v>
+        <v>11.080844437444306</v>
       </c>
       <c r="Y65" s="63" t="e">
         <f t="shared" si="100"/>
@@ -23372,93 +23548,93 @@
       <c r="B66" s="94" t="s">
         <v>37</v>
       </c>
-      <c r="C66" s="83" t="e">
+      <c r="C66" s="83">
         <f t="shared" ref="C66:AH66" si="105">C51/C57*1000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D66" s="63" t="e">
+        <v>1.4888854741902835</v>
+      </c>
+      <c r="D66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E66" s="39" t="e">
+        <v>3.1086344246093898</v>
+      </c>
+      <c r="E66" s="39">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F66" s="28" t="e">
+        <v>3.0705833709740515</v>
+      </c>
+      <c r="F66" s="28">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G66" s="63" t="e">
+        <v>7.8970018414403018</v>
+      </c>
+      <c r="G66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H66" s="63" t="e">
+        <v>2.9247820596998406</v>
+      </c>
+      <c r="H66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I66" s="28" t="e">
+        <v>4.1072424311601727</v>
+      </c>
+      <c r="I66" s="28">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J66" s="63" t="e">
+        <v>4.4883624700036799</v>
+      </c>
+      <c r="J66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K66" s="63" t="e">
+        <v>12.028961699535186</v>
+      </c>
+      <c r="K66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L66" s="28" t="e">
+        <v>2.502822728137466</v>
+      </c>
+      <c r="L66" s="28">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M66" s="63" t="e">
+        <v>16.001169497268261</v>
+      </c>
+      <c r="M66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N66" s="63" t="e">
+        <v>11.630114080400336</v>
+      </c>
+      <c r="N66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O66" s="28" t="e">
+        <v>3.2079051856571836</v>
+      </c>
+      <c r="O66" s="28">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P66" s="63" t="e">
+        <v>2.7331515387334759</v>
+      </c>
+      <c r="P66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q66" s="63" t="e">
+        <v>16.128947958707897</v>
+      </c>
+      <c r="Q66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R66" s="28" t="e">
+        <v>9.5729747454755127</v>
+      </c>
+      <c r="R66" s="28">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S66" s="63" t="e">
+        <v>9.128536666939965</v>
+      </c>
+      <c r="S66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T66" s="63" t="e">
+        <v>11.69543930945607</v>
+      </c>
+      <c r="T66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U66" s="28" t="e">
+        <v>5.2032711038009882</v>
+      </c>
+      <c r="U66" s="28">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V66" s="63" t="e">
+        <v>8.5293194033899677</v>
+      </c>
+      <c r="V66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W66" s="63" t="e">
+        <v>8.5811748869533027</v>
+      </c>
+      <c r="W66" s="63">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X66" s="28" t="e">
+        <v>12.694521193056117</v>
+      </c>
+      <c r="X66" s="28">
         <f t="shared" si="105"/>
-        <v>#DIV/0!</v>
+        <v>9.3201354135603509</v>
       </c>
       <c r="Y66" s="63" t="e">
         <f t="shared" si="105"/>
@@ -23932,93 +24108,93 @@
       <c r="B67" s="95" t="s">
         <v>37</v>
       </c>
-      <c r="C67" s="84" t="e">
+      <c r="C67" s="84">
         <f t="shared" ref="C67:AH67" si="110">C38-SUM(C64,C65,C66,C63)+$C$83</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D67" s="64" t="e">
+        <v>38.226442763351827</v>
+      </c>
+      <c r="D67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E67" s="41" t="e">
+        <v>11.973178422438096</v>
+      </c>
+      <c r="E67" s="41">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F67" s="48" t="e">
+        <v>18.909135682491296</v>
+      </c>
+      <c r="F67" s="48">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G67" s="64" t="e">
+        <v>25.219083525927573</v>
+      </c>
+      <c r="G67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H67" s="64" t="e">
+        <v>30.885296439049142</v>
+      </c>
+      <c r="H67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I67" s="48" t="e">
+        <v>7.9263871019937397</v>
+      </c>
+      <c r="I67" s="48">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J67" s="64" t="e">
+        <v>5.7787530376500129</v>
+      </c>
+      <c r="J67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K67" s="64" t="e">
+        <v>15.510635762992258</v>
+      </c>
+      <c r="K67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L67" s="48" t="e">
+        <v>2.7659177903944894</v>
+      </c>
+      <c r="L67" s="48">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M67" s="64" t="e">
+        <v>1.2801906890952637</v>
+      </c>
+      <c r="M67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N67" s="64" t="e">
+        <v>14.799197334849858</v>
+      </c>
+      <c r="N67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O67" s="48" t="e">
+        <v>8.7788156409354769</v>
+      </c>
+      <c r="O67" s="48">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P67" s="64" t="e">
+        <v>36.267809158832506</v>
+      </c>
+      <c r="P67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q67" s="64" t="e">
+        <v>19.39247000150301</v>
+      </c>
+      <c r="Q67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R67" s="48" t="e">
+        <v>31.589122016020568</v>
+      </c>
+      <c r="R67" s="48">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S67" s="64" t="e">
+        <v>18.624895618988891</v>
+      </c>
+      <c r="S67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T67" s="64" t="e">
+        <v>27.625914916150485</v>
+      </c>
+      <c r="T67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U67" s="48" t="e">
+        <v>37.134886431924187</v>
+      </c>
+      <c r="U67" s="48">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V67" s="64" t="e">
+        <v>19.183993007936461</v>
+      </c>
+      <c r="V67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W67" s="64" t="e">
+        <v>22.405264222508794</v>
+      </c>
+      <c r="W67" s="64">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X67" s="48" t="e">
+        <v>6.071122350997463</v>
+      </c>
+      <c r="X67" s="48">
         <f t="shared" si="110"/>
-        <v>#DIV/0!</v>
+        <v>14.62036516195294</v>
       </c>
       <c r="Y67" s="64" t="e">
         <f t="shared" si="110"/>
@@ -24492,93 +24668,93 @@
       <c r="B68" s="96" t="s">
         <v>37</v>
       </c>
-      <c r="C68" s="75" t="e">
+      <c r="C68" s="75">
         <f t="shared" ref="C68:AH68" si="115">SUM(C63:C67)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="D68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E68" s="13" t="e">
+        <v>50</v>
+      </c>
+      <c r="E68" s="13">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F68" s="12" t="e">
+        <v>50</v>
+      </c>
+      <c r="F68" s="12">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="G68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="H68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I68" s="12" t="e">
+        <v>50</v>
+      </c>
+      <c r="I68" s="12">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J68" s="55" t="e">
+        <v>50.000000000000007</v>
+      </c>
+      <c r="J68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="K68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L68" s="12" t="e">
+        <v>50</v>
+      </c>
+      <c r="L68" s="12">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="M68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N68" s="55" t="e">
+        <v>50.000000000000007</v>
+      </c>
+      <c r="N68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O68" s="12" t="e">
+        <v>50</v>
+      </c>
+      <c r="O68" s="12">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="P68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="Q68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R68" s="12" t="e">
+        <v>50</v>
+      </c>
+      <c r="R68" s="12">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="S68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="T68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U68" s="12" t="e">
+        <v>50</v>
+      </c>
+      <c r="U68" s="12">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="V68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W68" s="55" t="e">
+        <v>50</v>
+      </c>
+      <c r="W68" s="55">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X68" s="12" t="e">
+        <v>49.999999999999993</v>
+      </c>
+      <c r="X68" s="12">
         <f t="shared" si="115"/>
-        <v>#DIV/0!</v>
+        <v>50</v>
       </c>
       <c r="Y68" s="55" t="e">
         <f t="shared" si="115"/>
@@ -25050,93 +25226,93 @@
         <v>91</v>
       </c>
       <c r="B69" s="96"/>
-      <c r="C69" s="75" t="e">
+      <c r="C69" s="75" t="str">
         <f t="shared" ref="C69:AH69" si="120">IF(OR(C63&lt;0,C64&lt;0,C65&lt;0,C66&lt;0,C67&lt;0),"YES","NO")</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="D69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E69" s="13" t="e">
+        <v>NO</v>
+      </c>
+      <c r="E69" s="13" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F69" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="F69" s="12" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="G69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="H69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I69" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="I69" s="12" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="J69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="K69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L69" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="L69" s="12" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="M69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="N69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O69" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="O69" s="12" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="P69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="Q69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R69" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="R69" s="12" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="S69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="T69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U69" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="U69" s="12" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="V69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W69" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="W69" s="55" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X69" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="X69" s="12" t="str">
         <f t="shared" si="120"/>
-        <v>#DIV/0!</v>
+        <v>NO</v>
       </c>
       <c r="Y69" s="55" t="e">
         <f t="shared" si="120"/>
@@ -25608,93 +25784,93 @@
         <v>92</v>
       </c>
       <c r="B70" s="96"/>
-      <c r="C70" s="75" t="e">
+      <c r="C70" s="75" t="str">
         <f t="shared" ref="C70:AH70" si="125">IF(OR(C63&lt;1,C64&lt;1,C65&lt;1,C66&lt;1,C67&lt;1),"YES","NO")</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="D70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E70" s="13" t="e">
+        <v>NO</v>
+      </c>
+      <c r="E70" s="13" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F70" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="F70" s="12" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="G70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="H70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I70" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="I70" s="12" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="J70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="K70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L70" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="L70" s="12" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="M70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="N70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O70" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="O70" s="12" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="P70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="Q70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R70" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="R70" s="12" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="S70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="T70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U70" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="U70" s="12" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="V70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W70" s="55" t="e">
+        <v>NO</v>
+      </c>
+      <c r="W70" s="55" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X70" s="12" t="e">
+        <v>NO</v>
+      </c>
+      <c r="X70" s="12" t="str">
         <f t="shared" si="125"/>
-        <v>#DIV/0!</v>
+        <v>NO</v>
       </c>
       <c r="Y70" s="55" t="e">
         <f t="shared" si="125"/>
@@ -28137,93 +28313,93 @@
       <c r="B77" s="96" t="s">
         <v>37</v>
       </c>
-      <c r="C77" s="75" t="e">
+      <c r="C77" s="75">
         <f t="shared" ref="C77:AH77" si="145">SUM(C68,C75)-$C$83</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="D77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E77" s="13" t="e">
+        <v>100</v>
+      </c>
+      <c r="E77" s="13">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F77" s="12" t="e">
+        <v>100</v>
+      </c>
+      <c r="F77" s="12">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="G77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="H77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I77" s="12" t="e">
+        <v>100</v>
+      </c>
+      <c r="I77" s="12">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="J77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="K77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="K77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L77" s="12" t="e">
+        <v>100</v>
+      </c>
+      <c r="L77" s="12">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="M77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="M77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="N77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="N77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="O77" s="12" t="e">
+        <v>100</v>
+      </c>
+      <c r="O77" s="12">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="P77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="P77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="Q77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="Q77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="R77" s="12" t="e">
+        <v>100</v>
+      </c>
+      <c r="R77" s="12">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="S77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="S77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="T77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="U77" s="12" t="e">
+        <v>100</v>
+      </c>
+      <c r="U77" s="12">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="V77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="V77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="W77" s="55" t="e">
+        <v>100</v>
+      </c>
+      <c r="W77" s="55">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="X77" s="12" t="e">
+        <v>100</v>
+      </c>
+      <c r="X77" s="12">
         <f t="shared" si="145"/>
-        <v>#DIV/0!</v>
+        <v>100</v>
       </c>
       <c r="Y77" s="55" t="e">
         <f t="shared" si="145"/>

</xml_diff>